<commit_message>
conditionally removing the pop up on all the reports when raw data is submitted
</commit_message>
<xml_diff>
--- a/public/templates/CTScan_SingleTube_Sample.xlsx
+++ b/public/templates/CTScan_SingleTube_Sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECTS\anteso\anteso-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCEA6A7-8CC4-439C-B14C-ED7227A42A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF25B65D-8DB7-42C1-9160-09DFAF1D835B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="306">
   <si>
     <t>TEST: RADIATION PROFILE WIDTH FOR CT SCAN</t>
   </si>
@@ -438,15 +438,6 @@
   </si>
   <si>
     <t>0.5</t>
-  </si>
-  <si>
-    <t>TEST: ALIGNMENT OF TABLE/GANTRY</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>±2.0</t>
   </si>
   <si>
     <t>TEST: TABLE POSITION</t>
@@ -2549,6 +2540,474 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2564,24 +3023,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2606,9 +3047,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2617,453 +3055,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4701,47 +4692,26 @@
         <v>135</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>63</v>
-      </c>
-      <c r="B59" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>140</v>
-      </c>
-      <c r="B60" t="s">
-        <v>141</v>
-      </c>
-    </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B63" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C63" t="s">
         <v>2</v>
       </c>
       <c r="D63" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E63" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F63" t="s">
         <v>3</v>
@@ -4764,7 +4734,7 @@
         <v>41</v>
       </c>
       <c r="D64" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E64" t="s">
         <v>26</v>
@@ -4787,7 +4757,7 @@
         <v>44</v>
       </c>
       <c r="C65" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D65" t="s">
         <v>10</v>
@@ -4807,7 +4777,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
@@ -4815,29 +4785,29 @@
         <v>74</v>
       </c>
       <c r="B68" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C68" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B69" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C69" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B70" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C70" t="s">
         <v>138</v>
@@ -4845,18 +4815,18 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B71" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C71" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
@@ -4864,16 +4834,16 @@
         <v>115</v>
       </c>
       <c r="B74" t="s">
+        <v>156</v>
+      </c>
+      <c r="C74" t="s">
+        <v>157</v>
+      </c>
+      <c r="D74" t="s">
+        <v>158</v>
+      </c>
+      <c r="E74" t="s">
         <v>159</v>
-      </c>
-      <c r="C74" t="s">
-        <v>160</v>
-      </c>
-      <c r="D74" t="s">
-        <v>161</v>
-      </c>
-      <c r="E74" t="s">
-        <v>162</v>
       </c>
       <c r="F74" t="s">
         <v>4</v>
@@ -4890,19 +4860,19 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B75" t="s">
         <v>129</v>
       </c>
       <c r="C75" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D75" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E75" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="F75" t="s">
         <v>26</v>
@@ -4914,18 +4884,18 @@
         <v>138</v>
       </c>
       <c r="I75" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B76" t="s">
         <v>108</v>
       </c>
       <c r="C76" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D76" t="s">
         <v>10</v>
@@ -4949,7 +4919,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:M2 A5:M8 A4:H4 J4:M4 B3:M3 A12:M76 A9 C9:M9 A10 C10:M10 A11 C11:M11" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:M2 A5:M8 A4:H4 J4:M4 B3:M3 A12:M57 A9 C9:M9 A10 C10:M10 A11 C11:M11 A61:M76" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4979,40 +4949,40 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B1" s="342" t="s">
-        <v>170</v>
-      </c>
-      <c r="C1" s="342"/>
-      <c r="D1" s="342"/>
-      <c r="E1" s="342"/>
-      <c r="F1" s="342"/>
-      <c r="G1" s="342"/>
-      <c r="H1" s="342"/>
-      <c r="I1" s="342"/>
+        <v>166</v>
+      </c>
+      <c r="B1" s="175" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="346"/>
-      <c r="L1" s="346"/>
-      <c r="M1" s="346"/>
-      <c r="N1" s="222"/>
-      <c r="O1" s="222"/>
+      <c r="K1" s="177"/>
+      <c r="L1" s="177"/>
+      <c r="M1" s="177"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
       <c r="P1" s="3"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="B2" s="342" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="342"/>
-      <c r="D2" s="342"/>
-      <c r="E2" s="342"/>
-      <c r="F2" s="342"/>
-      <c r="G2" s="342"/>
-      <c r="H2" s="342"/>
-      <c r="I2" s="342"/>
+        <v>168</v>
+      </c>
+      <c r="B2" s="175" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="175"/>
+      <c r="D2" s="175"/>
+      <c r="E2" s="175"/>
+      <c r="F2" s="175"/>
+      <c r="G2" s="175"/>
+      <c r="H2" s="175"/>
+      <c r="I2" s="175"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -5022,16 +4992,16 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="342" t="s">
-        <v>173</v>
-      </c>
-      <c r="C3" s="342"/>
-      <c r="D3" s="342"/>
-      <c r="E3" s="342"/>
-      <c r="F3" s="342"/>
-      <c r="G3" s="342"/>
-      <c r="H3" s="342"/>
-      <c r="I3" s="342"/>
+      <c r="B3" s="175" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="175"/>
+      <c r="D3" s="175"/>
+      <c r="E3" s="175"/>
+      <c r="F3" s="175"/>
+      <c r="G3" s="175"/>
+      <c r="H3" s="175"/>
+      <c r="I3" s="175"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -5041,16 +5011,16 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B4" s="342"/>
-      <c r="C4" s="342"/>
-      <c r="D4" s="342"/>
-      <c r="E4" s="342"/>
-      <c r="F4" s="342"/>
-      <c r="G4" s="342"/>
-      <c r="H4" s="342"/>
-      <c r="I4" s="342"/>
+        <v>171</v>
+      </c>
+      <c r="B4" s="175"/>
+      <c r="C4" s="175"/>
+      <c r="D4" s="175"/>
+      <c r="E4" s="175"/>
+      <c r="F4" s="175"/>
+      <c r="G4" s="175"/>
+      <c r="H4" s="175"/>
+      <c r="I4" s="175"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -5060,22 +5030,22 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B5" s="342" t="s">
-        <v>176</v>
-      </c>
-      <c r="C5" s="342"/>
-      <c r="D5" s="342"/>
-      <c r="E5" s="342"/>
+        <v>172</v>
+      </c>
+      <c r="B5" s="175" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" s="175"/>
+      <c r="D5" s="175"/>
+      <c r="E5" s="175"/>
       <c r="F5" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="G5" s="345">
+        <v>174</v>
+      </c>
+      <c r="G5" s="176">
         <v>22.7</v>
       </c>
-      <c r="H5" s="345"/>
-      <c r="I5" s="345"/>
+      <c r="H5" s="176"/>
+      <c r="I5" s="176"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -5085,22 +5055,22 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="B6" s="342" t="s">
-        <v>179</v>
-      </c>
-      <c r="C6" s="342"/>
-      <c r="D6" s="342"/>
-      <c r="E6" s="342"/>
+        <v>175</v>
+      </c>
+      <c r="B6" s="175" t="s">
+        <v>176</v>
+      </c>
+      <c r="C6" s="175"/>
+      <c r="D6" s="175"/>
+      <c r="E6" s="175"/>
       <c r="F6" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="G6" s="345">
+        <v>177</v>
+      </c>
+      <c r="G6" s="176">
         <v>50.2</v>
       </c>
-      <c r="H6" s="345"/>
-      <c r="I6" s="345"/>
+      <c r="H6" s="176"/>
+      <c r="I6" s="176"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -5110,22 +5080,22 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="B7" s="342" t="s">
-        <v>182</v>
-      </c>
-      <c r="C7" s="342"/>
-      <c r="D7" s="342"/>
-      <c r="E7" s="342"/>
+        <v>178</v>
+      </c>
+      <c r="B7" s="175" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="175"/>
+      <c r="D7" s="175"/>
+      <c r="E7" s="175"/>
       <c r="F7" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G7" s="342" t="s">
-        <v>183</v>
-      </c>
-      <c r="H7" s="342"/>
-      <c r="I7" s="342"/>
+      <c r="G7" s="175" t="s">
+        <v>180</v>
+      </c>
+      <c r="H7" s="175"/>
+      <c r="I7" s="175"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -5134,18 +5104,18 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="B8" s="341">
+        <v>181</v>
+      </c>
+      <c r="B8" s="191">
         <v>46066</v>
       </c>
-      <c r="C8" s="342"/>
-      <c r="D8" s="342"/>
-      <c r="E8" s="342"/>
+      <c r="C8" s="175"/>
+      <c r="D8" s="175"/>
+      <c r="E8" s="175"/>
       <c r="F8" s="4"/>
-      <c r="G8" s="342"/>
-      <c r="H8" s="342"/>
-      <c r="I8" s="342"/>
+      <c r="G8" s="175"/>
+      <c r="H8" s="175"/>
+      <c r="I8" s="175"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -5154,14 +5124,14 @@
     </row>
     <row r="9" spans="1:27" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="336"/>
-      <c r="C9" s="336"/>
-      <c r="D9" s="336"/>
-      <c r="E9" s="336"/>
+      <c r="B9" s="184"/>
+      <c r="C9" s="184"/>
+      <c r="D9" s="184"/>
+      <c r="E9" s="184"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="336"/>
-      <c r="H9" s="336"/>
-      <c r="I9" s="336"/>
+      <c r="G9" s="184"/>
+      <c r="H9" s="184"/>
+      <c r="I9" s="184"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -5170,18 +5140,18 @@
     </row>
     <row r="10" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="343" t="s">
-        <v>186</v>
-      </c>
-      <c r="C10" s="343"/>
-      <c r="D10" s="343"/>
-      <c r="E10" s="343"/>
-      <c r="F10" s="343"/>
-      <c r="G10" s="343"/>
-      <c r="H10" s="343"/>
-      <c r="I10" s="344"/>
+        <v>182</v>
+      </c>
+      <c r="B10" s="192" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10" s="192"/>
+      <c r="D10" s="192"/>
+      <c r="E10" s="192"/>
+      <c r="F10" s="192"/>
+      <c r="G10" s="192"/>
+      <c r="H10" s="192"/>
+      <c r="I10" s="193"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -5189,39 +5159,39 @@
       <c r="N10" s="2"/>
     </row>
     <row r="11" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="183" t="s">
-        <v>187</v>
-      </c>
-      <c r="B11" s="184"/>
-      <c r="C11" s="185"/>
-      <c r="D11" s="184" t="s">
-        <v>188</v>
-      </c>
-      <c r="E11" s="184"/>
-      <c r="F11" s="184"/>
-      <c r="G11" s="184"/>
-      <c r="H11" s="184"/>
-      <c r="I11" s="185"/>
+      <c r="A11" s="194" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" s="195"/>
+      <c r="C11" s="196"/>
+      <c r="D11" s="195" t="s">
+        <v>185</v>
+      </c>
+      <c r="E11" s="195"/>
+      <c r="F11" s="195"/>
+      <c r="G11" s="195"/>
+      <c r="H11" s="195"/>
+      <c r="I11" s="196"/>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="9"/>
-      <c r="P11" s="331" t="s">
-        <v>189</v>
-      </c>
-      <c r="Q11" s="332"/>
-      <c r="R11" s="332"/>
-      <c r="S11" s="332"/>
-      <c r="T11" s="332"/>
-      <c r="U11" s="332"/>
-      <c r="V11" s="332"/>
-      <c r="W11" s="332"/>
-      <c r="X11" s="333"/>
+      <c r="P11" s="179" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q11" s="180"/>
+      <c r="R11" s="180"/>
+      <c r="S11" s="180"/>
+      <c r="T11" s="180"/>
+      <c r="U11" s="180"/>
+      <c r="V11" s="180"/>
+      <c r="W11" s="180"/>
+      <c r="X11" s="181"/>
     </row>
     <row r="12" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>4</v>
@@ -5230,22 +5200,22 @@
         <v>110</v>
       </c>
       <c r="D12" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G12" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="H12" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="I12" s="12" t="s">
         <v>192</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>193</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>195</v>
       </c>
       <c r="J12" s="9"/>
       <c r="K12" s="9"/>
@@ -5254,26 +5224,26 @@
         <v>65</v>
       </c>
       <c r="N12" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="P12" s="182" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q12" s="184" t="s">
+        <v>195</v>
+      </c>
+      <c r="R12" s="184"/>
+      <c r="S12" s="184"/>
+      <c r="T12" s="185" t="s">
         <v>196</v>
       </c>
-      <c r="P12" s="334" t="s">
+      <c r="U12" s="187" t="s">
         <v>197</v>
       </c>
-      <c r="Q12" s="336" t="s">
+      <c r="V12" s="185"/>
+      <c r="W12" s="5"/>
+      <c r="X12" s="189" t="s">
         <v>198</v>
-      </c>
-      <c r="R12" s="336"/>
-      <c r="S12" s="336"/>
-      <c r="T12" s="337" t="s">
-        <v>199</v>
-      </c>
-      <c r="U12" s="305" t="s">
-        <v>200</v>
-      </c>
-      <c r="V12" s="337"/>
-      <c r="W12" s="5"/>
-      <c r="X12" s="339" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -5312,7 +5282,7 @@
         <f>ROUND(F13,4)</f>
         <v>0.53200000000000003</v>
       </c>
-      <c r="P13" s="335"/>
+      <c r="P13" s="183"/>
       <c r="Q13" s="17">
         <f>B14</f>
         <v>10</v>
@@ -5325,11 +5295,11 @@
         <f>B22</f>
         <v>350</v>
       </c>
-      <c r="T13" s="338"/>
-      <c r="U13" s="216"/>
-      <c r="V13" s="338"/>
+      <c r="T13" s="186"/>
+      <c r="U13" s="188"/>
+      <c r="V13" s="186"/>
       <c r="W13" s="19"/>
-      <c r="X13" s="340"/>
+      <c r="X13" s="190"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="20">
@@ -5397,7 +5367,7 @@
         <v>0.70999999999999375</v>
       </c>
       <c r="Y14" s="28" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="Z14" s="29"/>
       <c r="AA14" s="29"/>
@@ -5498,7 +5468,7 @@
         <v>9.1636581420898438</v>
       </c>
       <c r="L16" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="M16">
         <f t="shared" si="1"/>
@@ -5588,7 +5558,7 @@
         <v>141.59</v>
       </c>
       <c r="S17" s="35" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="T17" s="36">
         <f>ROUND(AVERAGE(Q17:S17),2)</f>
@@ -5641,15 +5611,15 @@
         <f t="shared" si="0"/>
         <v>5.2999000000000001</v>
       </c>
-      <c r="P18" s="325" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q18" s="326"/>
-      <c r="R18" s="326"/>
-      <c r="S18" s="326"/>
-      <c r="T18" s="326"/>
-      <c r="U18" s="326"/>
-      <c r="V18" s="327"/>
+      <c r="P18" s="206" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q18" s="207"/>
+      <c r="R18" s="207"/>
+      <c r="S18" s="207"/>
+      <c r="T18" s="207"/>
+      <c r="U18" s="207"/>
+      <c r="V18" s="208"/>
       <c r="W18" s="40"/>
       <c r="X18" s="41"/>
     </row>
@@ -5689,13 +5659,13 @@
         <f t="shared" si="0"/>
         <v>5.3005000000000004</v>
       </c>
-      <c r="P19" s="289"/>
-      <c r="Q19" s="289"/>
-      <c r="R19" s="289"/>
-      <c r="S19" s="289"/>
-      <c r="T19" s="289"/>
-      <c r="U19" s="289"/>
-      <c r="V19" s="289"/>
+      <c r="P19" s="209"/>
+      <c r="Q19" s="209"/>
+      <c r="R19" s="209"/>
+      <c r="S19" s="209"/>
+      <c r="T19" s="209"/>
+      <c r="U19" s="209"/>
+      <c r="V19" s="209"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20" s="20">
@@ -5733,14 +5703,14 @@
         <f t="shared" si="0"/>
         <v>5.3002000000000002</v>
       </c>
-      <c r="P20" s="310" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q20" s="311"/>
-      <c r="R20" s="311"/>
-      <c r="S20" s="311"/>
-      <c r="T20" s="311"/>
-      <c r="U20" s="313"/>
+      <c r="P20" s="210" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q20" s="211"/>
+      <c r="R20" s="211"/>
+      <c r="S20" s="211"/>
+      <c r="T20" s="211"/>
+      <c r="U20" s="212"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="20">
@@ -5778,16 +5748,16 @@
         <f t="shared" si="0"/>
         <v>5.2969999999999997</v>
       </c>
-      <c r="P21" s="328" t="s">
-        <v>207</v>
-      </c>
-      <c r="Q21" s="329"/>
-      <c r="R21" s="330" t="s">
-        <v>208</v>
-      </c>
-      <c r="S21" s="329"/>
+      <c r="P21" s="213" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q21" s="214"/>
+      <c r="R21" s="215" t="s">
+        <v>205</v>
+      </c>
+      <c r="S21" s="214"/>
       <c r="T21" s="14" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="U21" s="43" t="s">
         <v>63</v>
@@ -5822,7 +5792,7 @@
         <v>9.1354408264160156</v>
       </c>
       <c r="J22" s="44" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="M22">
         <f t="shared" si="1"/>
@@ -5832,16 +5802,16 @@
         <f t="shared" si="0"/>
         <v>18.497399999999999</v>
       </c>
-      <c r="P22" s="316">
+      <c r="P22" s="197">
         <f>C14</f>
         <v>1</v>
       </c>
-      <c r="Q22" s="317"/>
-      <c r="R22" s="318">
+      <c r="Q22" s="198"/>
+      <c r="R22" s="199">
         <f>ROUND(E14/1000,4)</f>
         <v>1.0092000000000001</v>
       </c>
-      <c r="S22" s="318"/>
+      <c r="S22" s="199"/>
       <c r="T22" s="45">
         <f>ROUND(ABS(((R22-P22)/P22*100)),2)</f>
         <v>0.92</v>
@@ -5887,16 +5857,16 @@
         <f t="shared" si="0"/>
         <v>0.94920000000000004</v>
       </c>
-      <c r="P23" s="316">
+      <c r="P23" s="197">
         <f>C15</f>
         <v>2</v>
       </c>
-      <c r="Q23" s="317"/>
-      <c r="R23" s="318">
+      <c r="Q23" s="198"/>
+      <c r="R23" s="199">
         <f>ROUND(E15/1000,4)</f>
         <v>2.0093999999999999</v>
       </c>
-      <c r="S23" s="318"/>
+      <c r="S23" s="199"/>
       <c r="T23" s="45">
         <f>ROUND(ABS(((R23-P23)/P23*100)),2)</f>
         <v>0.47</v>
@@ -5942,16 +5912,16 @@
         <f t="shared" si="0"/>
         <v>9.4794</v>
       </c>
-      <c r="P24" s="316">
+      <c r="P24" s="197">
         <f>C16</f>
         <v>3</v>
       </c>
-      <c r="Q24" s="317"/>
-      <c r="R24" s="318">
+      <c r="Q24" s="198"/>
+      <c r="R24" s="199">
         <f>ROUND(E16/1000,4)</f>
         <v>3.0081000000000002</v>
       </c>
-      <c r="S24" s="318"/>
+      <c r="S24" s="199"/>
       <c r="T24" s="45">
         <f>ROUND(ABS(((R24-P24)/P24*100)),2)</f>
         <v>0.27</v>
@@ -5997,14 +5967,14 @@
         <f t="shared" si="0"/>
         <v>9.4793000000000003</v>
       </c>
-      <c r="P25" s="319" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q25" s="320"/>
-      <c r="R25" s="320"/>
-      <c r="S25" s="320"/>
-      <c r="T25" s="320"/>
-      <c r="U25" s="321"/>
+      <c r="P25" s="200" t="s">
+        <v>208</v>
+      </c>
+      <c r="Q25" s="201"/>
+      <c r="R25" s="201"/>
+      <c r="S25" s="201"/>
+      <c r="T25" s="201"/>
+      <c r="U25" s="202"/>
     </row>
     <row r="26" spans="1:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="20">
@@ -6079,20 +6049,20 @@
         <f t="shared" si="0"/>
         <v>9.4781999999999993</v>
       </c>
-      <c r="P27" s="322" t="s">
-        <v>212</v>
-      </c>
-      <c r="Q27" s="323"/>
-      <c r="R27" s="324"/>
+      <c r="P27" s="203" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q27" s="204"/>
+      <c r="R27" s="205"/>
       <c r="S27" s="47" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="T27" s="47">
         <f>A34</f>
         <v>120</v>
       </c>
       <c r="U27" s="47" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="V27" s="47"/>
       <c r="W27" s="47"/>
@@ -6138,23 +6108,23 @@
         <v>9.4741999999999997</v>
       </c>
       <c r="P28" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q28" s="187" t="s">
+        <v>212</v>
+      </c>
+      <c r="R28" s="187"/>
+      <c r="S28" s="187"/>
+      <c r="T28" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="U28" s="14" t="s">
         <v>214</v>
-      </c>
-      <c r="Q28" s="305" t="s">
-        <v>215</v>
-      </c>
-      <c r="R28" s="305"/>
-      <c r="S28" s="305"/>
-      <c r="T28" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="U28" s="14" t="s">
-        <v>217</v>
       </c>
       <c r="V28" s="5"/>
       <c r="W28" s="5"/>
       <c r="X28" s="43" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.3">
@@ -6186,7 +6156,7 @@
         <v>9.0879783630371094</v>
       </c>
       <c r="J29" s="44" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="M29">
         <f t="shared" si="1"/>
@@ -6216,13 +6186,13 @@
         <f>ROUND((AVERAGE(Q29:S29)/(P29*X27)),4)</f>
         <v>0.1457</v>
       </c>
-      <c r="U29" s="306">
+      <c r="U29" s="237">
         <f>ROUND((MAX(T29:T32)-MIN(T29:T32))/(MAX(T29:T32)+MIN(T29:T32)),4)</f>
         <v>1.4E-3</v>
       </c>
       <c r="V29" s="13"/>
       <c r="W29" s="5"/>
-      <c r="X29" s="308" t="str">
+      <c r="X29" s="239" t="str">
         <f>IF(U29&lt;0.1,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
@@ -6283,10 +6253,10 @@
         <f>ROUND((AVERAGE(Q30:S30)/(P30*X27)),4)</f>
         <v>0.14530000000000001</v>
       </c>
-      <c r="U30" s="306"/>
+      <c r="U30" s="237"/>
       <c r="V30" s="13"/>
       <c r="W30" s="5"/>
-      <c r="X30" s="308"/>
+      <c r="X30" s="239"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A31" s="20">
@@ -6344,10 +6314,10 @@
         <f>ROUND((AVERAGE(Q31:S31)/(P31*X27)),4)</f>
         <v>0.14549999999999999</v>
       </c>
-      <c r="U31" s="306"/>
+      <c r="U31" s="237"/>
       <c r="V31" s="13"/>
       <c r="W31" s="5"/>
-      <c r="X31" s="308"/>
+      <c r="X31" s="239"/>
     </row>
     <row r="32" spans="1:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="20">
@@ -6405,10 +6375,10 @@
         <f>ROUND((AVERAGE(Q32:S32)/(P32*X27)),4)</f>
         <v>0.1454</v>
       </c>
-      <c r="U32" s="307"/>
+      <c r="U32" s="238"/>
       <c r="V32" s="18"/>
       <c r="W32" s="19"/>
-      <c r="X32" s="309"/>
+      <c r="X32" s="240"/>
     </row>
     <row r="33" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="20">
@@ -6446,17 +6416,17 @@
         <f t="shared" si="0"/>
         <v>7.2878999999999996</v>
       </c>
-      <c r="P33" s="210" t="s">
-        <v>218</v>
-      </c>
-      <c r="Q33" s="211"/>
-      <c r="R33" s="211"/>
-      <c r="S33" s="211"/>
-      <c r="T33" s="211"/>
-      <c r="U33" s="211"/>
-      <c r="V33" s="211"/>
-      <c r="W33" s="211"/>
-      <c r="X33" s="212"/>
+      <c r="P33" s="220" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q33" s="221"/>
+      <c r="R33" s="221"/>
+      <c r="S33" s="221"/>
+      <c r="T33" s="221"/>
+      <c r="U33" s="221"/>
+      <c r="V33" s="221"/>
+      <c r="W33" s="221"/>
+      <c r="X33" s="222"/>
     </row>
     <row r="34" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="20">
@@ -6531,18 +6501,18 @@
         <f t="shared" si="0"/>
         <v>14.5259</v>
       </c>
-      <c r="P35" s="310" t="s">
-        <v>219</v>
-      </c>
-      <c r="Q35" s="311"/>
-      <c r="R35" s="311"/>
-      <c r="S35" s="311"/>
-      <c r="T35" s="311"/>
-      <c r="U35" s="311"/>
-      <c r="V35" s="312"/>
-      <c r="W35" s="312"/>
-      <c r="X35" s="312"/>
-      <c r="Y35" s="313"/>
+      <c r="P35" s="210" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q35" s="211"/>
+      <c r="R35" s="211"/>
+      <c r="S35" s="211"/>
+      <c r="T35" s="211"/>
+      <c r="U35" s="211"/>
+      <c r="V35" s="241"/>
+      <c r="W35" s="241"/>
+      <c r="X35" s="241"/>
+      <c r="Y35" s="212"/>
     </row>
     <row r="36" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="20">
@@ -6583,24 +6553,24 @@
       <c r="P36" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="Q36" s="314" t="s">
-        <v>215</v>
-      </c>
-      <c r="R36" s="314"/>
-      <c r="S36" s="314"/>
-      <c r="T36" s="314"/>
-      <c r="U36" s="315"/>
+      <c r="Q36" s="242" t="s">
+        <v>212</v>
+      </c>
+      <c r="R36" s="242"/>
+      <c r="S36" s="242"/>
+      <c r="T36" s="242"/>
+      <c r="U36" s="243"/>
       <c r="V36" s="18" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="W36" s="18" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="X36" s="17" t="s">
         <v>104</v>
       </c>
       <c r="Y36" s="57" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="37" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -6947,18 +6917,18 @@
         <f t="shared" si="0"/>
         <v>29.098600000000001</v>
       </c>
-      <c r="P41" s="210" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q41" s="211"/>
-      <c r="R41" s="211"/>
-      <c r="S41" s="211"/>
-      <c r="T41" s="211"/>
-      <c r="U41" s="211"/>
-      <c r="V41" s="211"/>
-      <c r="W41" s="211"/>
-      <c r="X41" s="211"/>
-      <c r="Y41" s="212"/>
+      <c r="P41" s="220" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q41" s="221"/>
+      <c r="R41" s="221"/>
+      <c r="S41" s="221"/>
+      <c r="T41" s="221"/>
+      <c r="U41" s="221"/>
+      <c r="V41" s="221"/>
+      <c r="W41" s="221"/>
+      <c r="X41" s="221"/>
+      <c r="Y41" s="222"/>
     </row>
     <row r="42" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="20">
@@ -6989,7 +6959,7 @@
         <v>9.0919656753540039</v>
       </c>
       <c r="J42" s="44" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="M42">
         <f t="shared" si="1"/>
@@ -7036,15 +7006,15 @@
         <f t="shared" si="0"/>
         <v>50.876800000000003</v>
       </c>
-      <c r="P43" s="180" t="s">
-        <v>223</v>
-      </c>
-      <c r="Q43" s="296"/>
+      <c r="P43" s="223" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q43" s="224"/>
       <c r="R43" s="72" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="S43" s="73" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -7084,7 +7054,7 @@
         <v>50.917000000000002</v>
       </c>
       <c r="P44" s="74" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="Q44" s="75">
         <f>A46</f>
@@ -7135,12 +7105,12 @@
         <f t="shared" si="0"/>
         <v>2.0246</v>
       </c>
-      <c r="P45" s="297" t="s">
-        <v>224</v>
-      </c>
-      <c r="Q45" s="298"/>
-      <c r="R45" s="298"/>
-      <c r="S45" s="299"/>
+      <c r="P45" s="225" t="s">
+        <v>221</v>
+      </c>
+      <c r="Q45" s="226"/>
+      <c r="R45" s="226"/>
+      <c r="S45" s="227"/>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A46" s="20">
@@ -7178,10 +7148,10 @@
         <f t="shared" si="0"/>
         <v>20.186800000000002</v>
       </c>
-      <c r="P46" s="297"/>
-      <c r="Q46" s="298"/>
-      <c r="R46" s="298"/>
-      <c r="S46" s="299"/>
+      <c r="P46" s="225"/>
+      <c r="Q46" s="226"/>
+      <c r="R46" s="226"/>
+      <c r="S46" s="227"/>
     </row>
     <row r="47" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="20">
@@ -7219,9 +7189,9 @@
         <f t="shared" si="0"/>
         <v>20.193899999999999</v>
       </c>
-      <c r="P47" s="229"/>
-      <c r="Q47" s="300"/>
-      <c r="R47" s="300"/>
+      <c r="P47" s="228"/>
+      <c r="Q47" s="229"/>
+      <c r="R47" s="229"/>
       <c r="S47" s="230"/>
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.3">
@@ -7364,7 +7334,7 @@
         <v>9.3486919403076172</v>
       </c>
       <c r="J51" s="44" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="M51">
         <f t="shared" si="1"/>
@@ -7436,62 +7406,62 @@
       <c r="J56" s="80"/>
     </row>
     <row r="57" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="301" t="s">
-        <v>225</v>
-      </c>
-      <c r="B57" s="302"/>
-      <c r="C57" s="302"/>
-      <c r="D57" s="302"/>
-      <c r="E57" s="302"/>
-      <c r="F57" s="302"/>
-      <c r="G57" s="302"/>
-      <c r="H57" s="302"/>
-      <c r="I57" s="303"/>
+      <c r="A57" s="231" t="s">
+        <v>222</v>
+      </c>
+      <c r="B57" s="232"/>
+      <c r="C57" s="232"/>
+      <c r="D57" s="232"/>
+      <c r="E57" s="232"/>
+      <c r="F57" s="232"/>
+      <c r="G57" s="232"/>
+      <c r="H57" s="232"/>
+      <c r="I57" s="233"/>
       <c r="J57" s="80"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="82"/>
       <c r="B58" s="83" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C58" s="84"/>
       <c r="D58" s="84" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E58" s="84"/>
       <c r="F58" s="84"/>
       <c r="G58" s="84" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H58" s="84" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I58" s="85"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="86"/>
       <c r="B59" s="87" t="s">
+        <v>227</v>
+      </c>
+      <c r="C59" s="87" t="s">
+        <v>228</v>
+      </c>
+      <c r="D59" s="87" t="s">
+        <v>229</v>
+      </c>
+      <c r="E59" s="87" t="s">
         <v>230</v>
       </c>
-      <c r="C59" s="87" t="s">
+      <c r="F59" s="87" t="s">
         <v>231</v>
       </c>
-      <c r="D59" s="87" t="s">
+      <c r="G59" s="87" t="s">
         <v>232</v>
       </c>
-      <c r="E59" s="87" t="s">
+      <c r="H59" s="234" t="s">
         <v>233</v>
       </c>
-      <c r="F59" s="87" t="s">
-        <v>234</v>
-      </c>
-      <c r="G59" s="87" t="s">
-        <v>235</v>
-      </c>
-      <c r="H59" s="291" t="s">
-        <v>236</v>
-      </c>
-      <c r="I59" s="292"/>
+      <c r="I59" s="235"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="86"/>
@@ -7502,7 +7472,7 @@
         <v>100</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -7510,71 +7480,71 @@
       <c r="F60" t="s">
         <v>84</v>
       </c>
-      <c r="H60" s="304">
+      <c r="H60" s="236">
         <v>18.12</v>
       </c>
-      <c r="I60" s="304"/>
+      <c r="I60" s="236"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="86"/>
       <c r="F61" t="s">
         <v>86</v>
       </c>
-      <c r="H61" s="287">
+      <c r="H61" s="248">
         <v>19.98</v>
       </c>
-      <c r="I61" s="287"/>
+      <c r="I61" s="248"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="86"/>
       <c r="F62" t="s">
         <v>89</v>
       </c>
-      <c r="H62" s="287">
+      <c r="H62" s="248">
         <v>18.7</v>
       </c>
-      <c r="I62" s="287"/>
+      <c r="I62" s="248"/>
       <c r="J62" s="88"/>
       <c r="K62" s="88"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="86"/>
       <c r="F63" t="s">
-        <v>238</v>
-      </c>
-      <c r="H63" s="287">
+        <v>235</v>
+      </c>
+      <c r="H63" s="248">
         <v>17.62</v>
       </c>
-      <c r="I63" s="287"/>
+      <c r="I63" s="248"/>
       <c r="J63" s="88"/>
       <c r="K63" s="88"/>
     </row>
     <row r="64" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="86"/>
       <c r="F64" t="s">
-        <v>239</v>
-      </c>
-      <c r="H64" s="290">
+        <v>236</v>
+      </c>
+      <c r="H64" s="249">
         <v>18.79</v>
       </c>
-      <c r="I64" s="290"/>
+      <c r="I64" s="249"/>
       <c r="J64" s="88"/>
       <c r="K64" s="88"/>
     </row>
     <row r="65" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="86"/>
-      <c r="B65" s="277" t="s">
-        <v>240</v>
-      </c>
-      <c r="C65" s="278"/>
+      <c r="B65" s="216" t="s">
+        <v>237</v>
+      </c>
+      <c r="C65" s="217"/>
       <c r="D65" s="91">
         <v>18.05</v>
       </c>
-      <c r="H65" s="294">
+      <c r="H65" s="218">
         <f>(H60/3)+(2/3*J65)</f>
         <v>18.555</v>
       </c>
-      <c r="I65" s="295"/>
+      <c r="I65" s="219"/>
       <c r="J65" s="92">
         <f>AVERAGE(H61:I64)</f>
         <v>18.772500000000001</v>
@@ -7589,11 +7559,11 @@
       <c r="G66" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="H66" s="242" t="str">
+      <c r="H66" s="244" t="str">
         <f>IF(K65&lt;20,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I66" s="244"/>
+      <c r="I66" s="245"/>
       <c r="J66" s="88"/>
       <c r="K66" s="88"/>
       <c r="P66" s="2"/>
@@ -7615,16 +7585,16 @@
     <row r="68" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A68" s="86"/>
       <c r="B68" s="44" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D68" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G68" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H68" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="I68" s="94"/>
       <c r="J68" s="88"/>
@@ -7637,31 +7607,31 @@
     <row r="69" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A69" s="86"/>
       <c r="B69" s="87" t="s">
+        <v>227</v>
+      </c>
+      <c r="C69" s="87" t="s">
+        <v>228</v>
+      </c>
+      <c r="D69" s="87" t="s">
+        <v>229</v>
+      </c>
+      <c r="E69" s="87" t="s">
         <v>230</v>
       </c>
-      <c r="C69" s="87" t="s">
+      <c r="F69" s="87" t="s">
         <v>231</v>
       </c>
-      <c r="D69" s="87" t="s">
+      <c r="G69" s="87" t="s">
         <v>232</v>
       </c>
-      <c r="E69" s="87" t="s">
+      <c r="H69" s="234" t="s">
         <v>233</v>
       </c>
-      <c r="F69" s="87" t="s">
-        <v>234</v>
-      </c>
-      <c r="G69" s="87" t="s">
-        <v>235</v>
-      </c>
-      <c r="H69" s="291" t="s">
-        <v>236</v>
-      </c>
-      <c r="I69" s="292"/>
-      <c r="P69" s="288"/>
-      <c r="Q69" s="288"/>
-      <c r="R69" s="289"/>
-      <c r="S69" s="289"/>
+      <c r="I69" s="235"/>
+      <c r="P69" s="246"/>
+      <c r="Q69" s="246"/>
+      <c r="R69" s="209"/>
+      <c r="S69" s="209"/>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A70" s="86"/>
@@ -7672,7 +7642,7 @@
         <v>100</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -7680,68 +7650,68 @@
       <c r="F70" t="s">
         <v>84</v>
       </c>
-      <c r="H70" s="293">
+      <c r="H70" s="247">
         <v>5.5410000000000004</v>
       </c>
-      <c r="I70" s="293"/>
-      <c r="P70" s="288"/>
-      <c r="Q70" s="288"/>
-      <c r="R70" s="289"/>
-      <c r="S70" s="289"/>
+      <c r="I70" s="247"/>
+      <c r="P70" s="246"/>
+      <c r="Q70" s="246"/>
+      <c r="R70" s="209"/>
+      <c r="S70" s="209"/>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A71" s="86"/>
       <c r="F71" t="s">
         <v>86</v>
       </c>
-      <c r="H71" s="287">
+      <c r="H71" s="248">
         <v>11.78</v>
       </c>
-      <c r="I71" s="287"/>
-      <c r="P71" s="288"/>
-      <c r="Q71" s="288"/>
-      <c r="R71" s="289"/>
-      <c r="S71" s="289"/>
+      <c r="I71" s="248"/>
+      <c r="P71" s="246"/>
+      <c r="Q71" s="246"/>
+      <c r="R71" s="209"/>
+      <c r="S71" s="209"/>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A72" s="86"/>
       <c r="F72" t="s">
         <v>89</v>
       </c>
-      <c r="H72" s="287">
+      <c r="H72" s="248">
         <v>12.39</v>
       </c>
-      <c r="I72" s="287"/>
-      <c r="P72" s="288"/>
-      <c r="Q72" s="288"/>
-      <c r="R72" s="289"/>
-      <c r="S72" s="289"/>
+      <c r="I72" s="248"/>
+      <c r="P72" s="246"/>
+      <c r="Q72" s="246"/>
+      <c r="R72" s="209"/>
+      <c r="S72" s="209"/>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A73" s="86"/>
       <c r="F73" t="s">
-        <v>238</v>
-      </c>
-      <c r="H73" s="287">
+        <v>235</v>
+      </c>
+      <c r="H73" s="248">
         <v>11.21</v>
       </c>
-      <c r="I73" s="287"/>
+      <c r="I73" s="248"/>
       <c r="J73" s="88"/>
       <c r="K73" s="88"/>
-      <c r="P73" s="288"/>
-      <c r="Q73" s="288"/>
-      <c r="R73" s="289"/>
-      <c r="S73" s="289"/>
+      <c r="P73" s="246"/>
+      <c r="Q73" s="246"/>
+      <c r="R73" s="209"/>
+      <c r="S73" s="209"/>
     </row>
     <row r="74" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A74" s="86"/>
       <c r="F74" t="s">
-        <v>239</v>
-      </c>
-      <c r="H74" s="290">
+        <v>236</v>
+      </c>
+      <c r="H74" s="249">
         <v>12.75</v>
       </c>
-      <c r="I74" s="290"/>
+      <c r="I74" s="249"/>
       <c r="J74" s="95">
         <f>AVERAGE(H71:I74)</f>
         <v>12.032500000000001</v>
@@ -7750,28 +7720,28 @@
         <f>ABS(H75-D75)/D75*100</f>
         <v>4.2097852868708063</v>
       </c>
-      <c r="P74" s="288"/>
-      <c r="Q74" s="288"/>
-      <c r="R74" s="289"/>
-      <c r="S74" s="289"/>
+      <c r="P74" s="246"/>
+      <c r="Q74" s="246"/>
+      <c r="R74" s="209"/>
+      <c r="S74" s="209"/>
     </row>
     <row r="75" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="96"/>
-      <c r="B75" s="277" t="s">
-        <v>240</v>
-      </c>
-      <c r="C75" s="278"/>
+      <c r="B75" s="216" t="s">
+        <v>237</v>
+      </c>
+      <c r="C75" s="217"/>
       <c r="D75" s="91">
         <v>9.4700000000000006</v>
       </c>
       <c r="E75" s="97"/>
       <c r="F75" s="97"/>
       <c r="G75" s="97"/>
-      <c r="H75" s="279">
+      <c r="H75" s="260">
         <f>(H70/3)+(2/3*J74)</f>
         <v>9.868666666666666</v>
       </c>
-      <c r="I75" s="280"/>
+      <c r="I75" s="261"/>
       <c r="J75" s="98"/>
       <c r="K75" s="98"/>
     </row>
@@ -7779,24 +7749,24 @@
       <c r="G76" s="99" t="s">
         <v>63</v>
       </c>
-      <c r="H76" s="180" t="str">
+      <c r="H76" s="223" t="str">
         <f>IF(K74&lt;20,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I76" s="182"/>
+      <c r="I76" s="262"/>
     </row>
     <row r="77" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="281" t="s">
-        <v>243</v>
-      </c>
-      <c r="B77" s="282"/>
-      <c r="C77" s="282"/>
-      <c r="D77" s="282"/>
-      <c r="E77" s="282"/>
-      <c r="F77" s="282"/>
-      <c r="G77" s="282"/>
-      <c r="H77" s="282"/>
-      <c r="I77" s="283"/>
+      <c r="A77" s="263" t="s">
+        <v>240</v>
+      </c>
+      <c r="B77" s="264"/>
+      <c r="C77" s="264"/>
+      <c r="D77" s="264"/>
+      <c r="E77" s="264"/>
+      <c r="F77" s="264"/>
+      <c r="G77" s="264"/>
+      <c r="H77" s="264"/>
+      <c r="I77" s="265"/>
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.3">
       <c r="G78" s="9"/>
@@ -7809,16 +7779,16 @@
       <c r="I79" s="100"/>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A80" s="180" t="s">
-        <v>244</v>
-      </c>
-      <c r="B80" s="181"/>
-      <c r="C80" s="181"/>
+      <c r="A80" s="223" t="s">
+        <v>241</v>
+      </c>
+      <c r="B80" s="266"/>
+      <c r="C80" s="266"/>
       <c r="D80" s="47" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E80" s="48" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="G80" s="88"/>
       <c r="H80" s="88"/>
@@ -7830,20 +7800,20 @@
       <c r="A81" s="101" t="s">
         <v>65</v>
       </c>
-      <c r="B81" s="284" t="s">
+      <c r="B81" s="267" t="s">
         <v>4</v>
       </c>
-      <c r="C81" s="285"/>
+      <c r="C81" s="268"/>
       <c r="D81" s="102" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E81" s="103">
         <f t="array" ref="E81">INDEX($J$82:$J$84,MATCH(E80,$I$82:$I$84,0),0)</f>
         <v>0.5</v>
       </c>
       <c r="G81" s="88"/>
-      <c r="H81" s="286"/>
-      <c r="I81" s="286"/>
+      <c r="H81" s="269"/>
+      <c r="I81" s="269"/>
       <c r="J81" s="88"/>
       <c r="K81" s="88"/>
     </row>
@@ -7851,18 +7821,18 @@
       <c r="A82" s="104">
         <v>140</v>
       </c>
-      <c r="B82" s="268">
+      <c r="B82" s="250">
         <v>15</v>
       </c>
-      <c r="C82" s="268"/>
-      <c r="D82" s="269" t="s">
-        <v>248</v>
+      <c r="C82" s="250"/>
+      <c r="D82" s="251" t="s">
+        <v>245</v>
       </c>
       <c r="E82" s="106"/>
       <c r="G82" s="88"/>
       <c r="H82" s="107"/>
       <c r="I82" s="108" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="J82" s="109">
         <v>0.42</v>
@@ -7871,15 +7841,15 @@
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" s="50" t="s">
-        <v>250</v>
-      </c>
-      <c r="B83" s="272" t="s">
-        <v>251</v>
-      </c>
-      <c r="C83" s="263"/>
-      <c r="D83" s="270"/>
+        <v>247</v>
+      </c>
+      <c r="B83" s="254" t="s">
+        <v>248</v>
+      </c>
+      <c r="C83" s="255"/>
+      <c r="D83" s="252"/>
       <c r="E83" s="46" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F83" s="110" t="s">
         <v>63</v>
@@ -7887,7 +7857,7 @@
       <c r="G83" s="88"/>
       <c r="H83" s="107"/>
       <c r="I83" s="108" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J83" s="109">
         <v>0.5</v>
@@ -7898,11 +7868,11 @@
       <c r="A84" s="50">
         <v>1.25</v>
       </c>
-      <c r="B84" s="273">
+      <c r="B84" s="256">
         <v>2.8</v>
       </c>
-      <c r="C84" s="273"/>
-      <c r="D84" s="270"/>
+      <c r="C84" s="256"/>
+      <c r="D84" s="252"/>
       <c r="E84" s="111">
         <f>B84*E81</f>
         <v>1.4</v>
@@ -7917,7 +7887,7 @@
       </c>
       <c r="H84" s="88"/>
       <c r="I84" s="112" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="J84" s="109">
         <v>0.5</v>
@@ -7928,11 +7898,11 @@
       <c r="A85" s="50">
         <v>2.5</v>
       </c>
-      <c r="B85" s="274">
+      <c r="B85" s="257">
         <v>5</v>
       </c>
-      <c r="C85" s="275"/>
-      <c r="D85" s="270"/>
+      <c r="C85" s="258"/>
+      <c r="D85" s="252"/>
       <c r="E85" s="111">
         <f>B85*E81</f>
         <v>2.5</v>
@@ -7954,11 +7924,11 @@
       <c r="A86" s="113">
         <v>5</v>
       </c>
-      <c r="B86" s="276">
+      <c r="B86" s="259">
         <v>9.8000000000000007</v>
       </c>
-      <c r="C86" s="276"/>
-      <c r="D86" s="271"/>
+      <c r="C86" s="259"/>
+      <c r="D86" s="253"/>
       <c r="E86" s="115">
         <f>B86*E81</f>
         <v>4.9000000000000004</v>
@@ -7977,14 +7947,14 @@
       <c r="K86" s="88"/>
     </row>
     <row r="87" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="254" t="s">
-        <v>254</v>
-      </c>
-      <c r="B87" s="255"/>
-      <c r="C87" s="255"/>
-      <c r="D87" s="255"/>
-      <c r="E87" s="255"/>
-      <c r="F87" s="256"/>
+      <c r="A87" s="282" t="s">
+        <v>251</v>
+      </c>
+      <c r="B87" s="283"/>
+      <c r="C87" s="283"/>
+      <c r="D87" s="283"/>
+      <c r="E87" s="283"/>
+      <c r="F87" s="284"/>
       <c r="G87" s="88"/>
       <c r="H87" s="88"/>
       <c r="I87" s="88"/>
@@ -7992,12 +7962,12 @@
       <c r="K87" s="88"/>
     </row>
     <row r="88" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="257"/>
-      <c r="B88" s="258"/>
-      <c r="C88" s="258"/>
-      <c r="D88" s="258"/>
-      <c r="E88" s="258"/>
-      <c r="F88" s="259"/>
+      <c r="A88" s="285"/>
+      <c r="B88" s="286"/>
+      <c r="C88" s="286"/>
+      <c r="D88" s="286"/>
+      <c r="E88" s="286"/>
+      <c r="F88" s="287"/>
       <c r="G88" s="88"/>
       <c r="H88" s="88"/>
       <c r="I88" s="88"/>
@@ -8012,11 +7982,11 @@
       <c r="B90" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="C90" s="181" t="s">
-        <v>255</v>
-      </c>
-      <c r="D90" s="181"/>
-      <c r="E90" s="182"/>
+      <c r="C90" s="266" t="s">
+        <v>252</v>
+      </c>
+      <c r="D90" s="266"/>
+      <c r="E90" s="262"/>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91" s="118">
@@ -8028,37 +7998,37 @@
       <c r="C91" s="119" t="s">
         <v>134</v>
       </c>
-      <c r="D91" s="260">
+      <c r="D91" s="288">
         <v>107</v>
       </c>
-      <c r="E91" s="261"/>
+      <c r="E91" s="289"/>
       <c r="F91" s="120" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A92" s="262" t="s">
-        <v>256</v>
-      </c>
-      <c r="B92" s="263"/>
-      <c r="C92" s="264">
+      <c r="A92" s="290" t="s">
+        <v>253</v>
+      </c>
+      <c r="B92" s="255"/>
+      <c r="C92" s="291">
         <v>3</v>
       </c>
-      <c r="D92" s="264"/>
-      <c r="E92" s="264"/>
+      <c r="D92" s="291"/>
+      <c r="E92" s="291"/>
       <c r="F92" s="121" t="str">
         <f>IF(C92&lt;=5,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A93" s="265" t="s">
-        <v>257</v>
-      </c>
-      <c r="B93" s="266"/>
-      <c r="C93" s="266"/>
-      <c r="D93" s="266"/>
-      <c r="E93" s="267"/>
+      <c r="A93" s="292" t="s">
+        <v>254</v>
+      </c>
+      <c r="B93" s="293"/>
+      <c r="C93" s="293"/>
+      <c r="D93" s="293"/>
+      <c r="E93" s="294"/>
     </row>
     <row r="94" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A94" s="122"/>
@@ -8074,11 +8044,11 @@
       <c r="B95" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="C95" s="242" t="s">
-        <v>258</v>
-      </c>
-      <c r="D95" s="243"/>
-      <c r="E95" s="244"/>
+      <c r="C95" s="244" t="s">
+        <v>255</v>
+      </c>
+      <c r="D95" s="270"/>
+      <c r="E95" s="245"/>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96" s="118">
@@ -8090,44 +8060,44 @@
       <c r="C96" s="127" t="s">
         <v>134</v>
       </c>
-      <c r="D96" s="245">
+      <c r="D96" s="271">
         <v>3691</v>
       </c>
-      <c r="E96" s="246"/>
+      <c r="E96" s="272"/>
       <c r="F96" s="120" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="97" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="247" t="s">
-        <v>256</v>
-      </c>
-      <c r="B97" s="248"/>
-      <c r="C97" s="249">
+      <c r="A97" s="273" t="s">
+        <v>253</v>
+      </c>
+      <c r="B97" s="274"/>
+      <c r="C97" s="275">
         <v>6.25</v>
       </c>
-      <c r="D97" s="249"/>
-      <c r="E97" s="249"/>
+      <c r="D97" s="275"/>
+      <c r="E97" s="275"/>
       <c r="F97" s="121" t="str">
         <f>IF(C97&gt;=3.12,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A98" s="250" t="s">
-        <v>259</v>
-      </c>
-      <c r="B98" s="251"/>
-      <c r="C98" s="251"/>
-      <c r="D98" s="251"/>
-      <c r="E98" s="252"/>
+      <c r="A98" s="276" t="s">
+        <v>256</v>
+      </c>
+      <c r="B98" s="277"/>
+      <c r="C98" s="277"/>
+      <c r="D98" s="277"/>
+      <c r="E98" s="278"/>
     </row>
     <row r="99" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="225"/>
-      <c r="B99" s="253"/>
-      <c r="C99" s="253"/>
-      <c r="D99" s="253"/>
-      <c r="E99" s="226"/>
+      <c r="A99" s="279"/>
+      <c r="B99" s="280"/>
+      <c r="C99" s="280"/>
+      <c r="D99" s="280"/>
+      <c r="E99" s="281"/>
     </row>
     <row r="100" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="128"/>
@@ -8137,28 +8107,28 @@
       <c r="E100" s="128"/>
     </row>
     <row r="101" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="242" t="s">
-        <v>260</v>
-      </c>
-      <c r="B101" s="243"/>
-      <c r="C101" s="243"/>
-      <c r="D101" s="243"/>
-      <c r="E101" s="243"/>
-      <c r="F101" s="243"/>
-      <c r="G101" s="243"/>
-      <c r="H101" s="243"/>
-      <c r="I101" s="243"/>
-      <c r="J101" s="244"/>
+      <c r="A101" s="244" t="s">
+        <v>257</v>
+      </c>
+      <c r="B101" s="270"/>
+      <c r="C101" s="270"/>
+      <c r="D101" s="270"/>
+      <c r="E101" s="270"/>
+      <c r="F101" s="270"/>
+      <c r="G101" s="270"/>
+      <c r="H101" s="270"/>
+      <c r="I101" s="270"/>
+      <c r="J101" s="245"/>
     </row>
     <row r="102" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A102" s="89" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B102" s="90" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C102" s="77" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D102" s="84"/>
       <c r="E102" s="89" t="s">
@@ -8168,11 +8138,11 @@
         <v>500</v>
       </c>
       <c r="G102" s="129" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="H102" s="130"/>
-      <c r="I102" s="219"/>
-      <c r="J102" s="220"/>
+      <c r="I102" s="300"/>
+      <c r="J102" s="301"/>
     </row>
     <row r="103" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A103" s="131">
@@ -8184,92 +8154,92 @@
       <c r="C103" s="133">
         <v>1</v>
       </c>
-      <c r="D103" s="221"/>
-      <c r="E103" s="222"/>
-      <c r="F103" s="222"/>
-      <c r="G103" s="223" t="s">
+      <c r="D103" s="302"/>
+      <c r="E103" s="178"/>
+      <c r="F103" s="178"/>
+      <c r="G103" s="303" t="s">
+        <v>261</v>
+      </c>
+      <c r="H103" s="304"/>
+      <c r="I103" s="305" t="s">
+        <v>262</v>
+      </c>
+      <c r="J103" s="306"/>
+      <c r="K103" s="307" t="s">
+        <v>63</v>
+      </c>
+      <c r="L103" s="308"/>
+    </row>
+    <row r="104" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A104" s="311" t="s">
+        <v>124</v>
+      </c>
+      <c r="B104" s="134" t="s">
+        <v>263</v>
+      </c>
+      <c r="C104" s="135" t="s">
         <v>264</v>
       </c>
-      <c r="H103" s="224"/>
-      <c r="I103" s="227" t="s">
+      <c r="D104" s="135" t="s">
         <v>265</v>
       </c>
-      <c r="J103" s="228"/>
-      <c r="K103" s="231" t="s">
-        <v>63</v>
-      </c>
-      <c r="L103" s="232"/>
-    </row>
-    <row r="104" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A104" s="235" t="s">
-        <v>124</v>
-      </c>
-      <c r="B104" s="134" t="s">
+      <c r="E104" s="136" t="s">
         <v>266</v>
       </c>
-      <c r="C104" s="135" t="s">
+      <c r="F104" s="135" t="s">
         <v>267</v>
       </c>
-      <c r="D104" s="135" t="s">
-        <v>268</v>
-      </c>
-      <c r="E104" s="136" t="s">
-        <v>269</v>
-      </c>
-      <c r="F104" s="135" t="s">
-        <v>270</v>
-      </c>
-      <c r="G104" s="225"/>
-      <c r="H104" s="226"/>
-      <c r="I104" s="229"/>
+      <c r="G104" s="279"/>
+      <c r="H104" s="281"/>
+      <c r="I104" s="228"/>
       <c r="J104" s="230"/>
-      <c r="K104" s="233"/>
-      <c r="L104" s="234"/>
+      <c r="K104" s="309"/>
+      <c r="L104" s="310"/>
     </row>
     <row r="105" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A105" s="194"/>
+      <c r="A105" s="312"/>
       <c r="B105" s="138"/>
       <c r="C105" s="139"/>
       <c r="D105" s="139"/>
       <c r="E105" s="140"/>
       <c r="F105" s="141" t="s">
-        <v>159</v>
-      </c>
-      <c r="G105" s="236">
+        <v>156</v>
+      </c>
+      <c r="G105" s="313">
         <f>ROUND(F102*MAX(B105:E105)/(60*B103),3)</f>
         <v>0</v>
       </c>
-      <c r="H105" s="237"/>
-      <c r="I105" s="238">
+      <c r="H105" s="314"/>
+      <c r="I105" s="315">
         <f>ROUND(8.33*MAX(B105:F105)/(B103*114),3)</f>
         <v>0</v>
       </c>
-      <c r="J105" s="239"/>
-      <c r="K105" s="240" t="str">
+      <c r="J105" s="316"/>
+      <c r="K105" s="317" t="str">
         <f>IF(I105&lt;=1,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="L105" s="241"/>
+      <c r="L105" s="318"/>
     </row>
     <row r="106" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A106" s="210" t="s">
-        <v>271</v>
-      </c>
-      <c r="B106" s="211"/>
-      <c r="C106" s="211"/>
-      <c r="D106" s="211"/>
-      <c r="E106" s="211"/>
-      <c r="F106" s="211"/>
-      <c r="G106" s="211"/>
-      <c r="H106" s="211"/>
-      <c r="I106" s="211"/>
-      <c r="J106" s="211"/>
-      <c r="K106" s="211"/>
-      <c r="L106" s="212"/>
+      <c r="A106" s="220" t="s">
+        <v>268</v>
+      </c>
+      <c r="B106" s="221"/>
+      <c r="C106" s="221"/>
+      <c r="D106" s="221"/>
+      <c r="E106" s="221"/>
+      <c r="F106" s="221"/>
+      <c r="G106" s="221"/>
+      <c r="H106" s="221"/>
+      <c r="I106" s="221"/>
+      <c r="J106" s="221"/>
+      <c r="K106" s="221"/>
+      <c r="L106" s="222"/>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="109" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -8281,10 +8251,10 @@
         <v>4</v>
       </c>
       <c r="C110" s="47" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D110" s="48" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -8314,49 +8284,49 @@
       <c r="I112" s="88"/>
     </row>
     <row r="113" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="213" t="s">
+      <c r="A113" s="295" t="s">
         <v>115</v>
       </c>
-      <c r="B113" s="214"/>
-      <c r="C113" s="214"/>
-      <c r="D113" s="214"/>
-      <c r="E113" s="214" t="s">
+      <c r="B113" s="296"/>
+      <c r="C113" s="296"/>
+      <c r="D113" s="296"/>
+      <c r="E113" s="296" t="s">
+        <v>272</v>
+      </c>
+      <c r="F113" s="296"/>
+      <c r="G113" s="296" t="s">
+        <v>273</v>
+      </c>
+      <c r="H113" s="296" t="s">
+        <v>63</v>
+      </c>
+      <c r="I113" s="298" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="114" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A114" s="297"/>
+      <c r="B114" s="188"/>
+      <c r="C114" s="188"/>
+      <c r="D114" s="188"/>
+      <c r="E114" s="188"/>
+      <c r="F114" s="188"/>
+      <c r="G114" s="188"/>
+      <c r="H114" s="188"/>
+      <c r="I114" s="299"/>
+    </row>
+    <row r="115" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="326" t="s">
         <v>275</v>
       </c>
-      <c r="F113" s="214"/>
-      <c r="G113" s="214" t="s">
-        <v>276</v>
-      </c>
-      <c r="H113" s="214" t="s">
-        <v>63</v>
-      </c>
-      <c r="I113" s="217" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="114" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="215"/>
-      <c r="B114" s="216"/>
-      <c r="C114" s="216"/>
-      <c r="D114" s="216"/>
-      <c r="E114" s="216"/>
-      <c r="F114" s="216"/>
-      <c r="G114" s="216"/>
-      <c r="H114" s="216"/>
-      <c r="I114" s="218"/>
-    </row>
-    <row r="115" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="205" t="s">
-        <v>278</v>
-      </c>
-      <c r="B115" s="206"/>
-      <c r="C115" s="206"/>
-      <c r="D115" s="206"/>
+      <c r="B115" s="327"/>
+      <c r="C115" s="327"/>
+      <c r="D115" s="327"/>
       <c r="E115" s="144">
         <v>2.7E-2</v>
       </c>
       <c r="F115" s="145" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G115" s="146">
         <f>ROUND((E115*D111)/(60*B111),3)</f>
@@ -8366,22 +8336,22 @@
         <f>IF(E115&lt;=2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I115" s="207" t="s">
-        <v>279</v>
+      <c r="I115" s="328" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="116" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="201" t="s">
-        <v>280</v>
-      </c>
-      <c r="B116" s="202"/>
-      <c r="C116" s="202"/>
-      <c r="D116" s="202"/>
+      <c r="A116" s="322" t="s">
+        <v>277</v>
+      </c>
+      <c r="B116" s="323"/>
+      <c r="C116" s="323"/>
+      <c r="D116" s="323"/>
       <c r="E116" s="148">
         <v>4.3999999999999997E-2</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G116" s="45">
         <f>ROUND((E116*D111)/(60*B111),3)</f>
@@ -8391,20 +8361,20 @@
         <f t="shared" ref="H116:H119" si="11">IF(E116&lt;=2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I116" s="208"/>
+      <c r="I116" s="329"/>
     </row>
     <row r="117" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="201" t="s">
-        <v>281</v>
-      </c>
-      <c r="B117" s="202"/>
-      <c r="C117" s="202"/>
-      <c r="D117" s="202"/>
+      <c r="A117" s="322" t="s">
+        <v>278</v>
+      </c>
+      <c r="B117" s="323"/>
+      <c r="C117" s="323"/>
+      <c r="D117" s="323"/>
       <c r="E117" s="148">
         <v>3.4000000000000002E-2</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G117" s="45">
         <f>ROUND((E117*D111)/(60*B111),3)</f>
@@ -8414,20 +8384,20 @@
         <f t="shared" si="11"/>
         <v>Pass</v>
       </c>
-      <c r="I117" s="208"/>
+      <c r="I117" s="329"/>
     </row>
     <row r="118" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="201" t="s">
-        <v>282</v>
-      </c>
-      <c r="B118" s="202"/>
-      <c r="C118" s="202"/>
-      <c r="D118" s="202"/>
+      <c r="A118" s="322" t="s">
+        <v>279</v>
+      </c>
+      <c r="B118" s="323"/>
+      <c r="C118" s="323"/>
+      <c r="D118" s="323"/>
       <c r="E118" s="148">
         <v>0.04</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G118" s="45">
         <f>ROUND((E118*D111)/(60*B111),3)</f>
@@ -8437,20 +8407,20 @@
         <f t="shared" si="11"/>
         <v>Pass</v>
       </c>
-      <c r="I118" s="208"/>
+      <c r="I118" s="329"/>
     </row>
     <row r="119" spans="1:15" ht="14.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A119" s="203" t="s">
-        <v>283</v>
-      </c>
-      <c r="B119" s="204"/>
-      <c r="C119" s="204"/>
-      <c r="D119" s="204"/>
+      <c r="A119" s="324" t="s">
+        <v>280</v>
+      </c>
+      <c r="B119" s="325"/>
+      <c r="C119" s="325"/>
+      <c r="D119" s="325"/>
       <c r="E119" s="150">
         <v>3.2000000000000001E-2</v>
       </c>
       <c r="F119" s="151" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G119" s="152">
         <f>ROUND((E119*D111)/(60*B111),3)</f>
@@ -8460,20 +8430,20 @@
         <f t="shared" si="11"/>
         <v>Pass</v>
       </c>
-      <c r="I119" s="209"/>
+      <c r="I119" s="330"/>
     </row>
     <row r="120" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="196" t="s">
-        <v>284</v>
-      </c>
-      <c r="B120" s="197"/>
-      <c r="C120" s="197"/>
-      <c r="D120" s="197"/>
+      <c r="A120" s="345" t="s">
+        <v>281</v>
+      </c>
+      <c r="B120" s="346"/>
+      <c r="C120" s="346"/>
+      <c r="D120" s="346"/>
       <c r="E120" s="154">
         <v>0.106</v>
       </c>
       <c r="F120" s="155" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G120" s="156">
         <f>ROUND((E120*D111)/(60*B111),3)</f>
@@ -8483,22 +8453,22 @@
         <f>IF(E120&lt;=0.2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I120" s="198" t="s">
-        <v>285</v>
+      <c r="I120" s="319" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="121" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="201" t="s">
-        <v>286</v>
-      </c>
-      <c r="B121" s="202"/>
-      <c r="C121" s="202"/>
-      <c r="D121" s="202"/>
+      <c r="A121" s="322" t="s">
+        <v>283</v>
+      </c>
+      <c r="B121" s="323"/>
+      <c r="C121" s="323"/>
+      <c r="D121" s="323"/>
       <c r="E121" s="148">
         <v>3.7999999999999999E-2</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G121" s="45">
         <f>ROUND((E121*D111)/(60*B111),3)</f>
@@ -8508,20 +8478,20 @@
         <f t="shared" ref="H121:H123" si="12">IF(E121&lt;=0.2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I121" s="199"/>
+      <c r="I121" s="320"/>
     </row>
     <row r="122" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="201" t="s">
-        <v>287</v>
-      </c>
-      <c r="B122" s="202"/>
-      <c r="C122" s="202"/>
-      <c r="D122" s="202"/>
+      <c r="A122" s="322" t="s">
+        <v>284</v>
+      </c>
+      <c r="B122" s="323"/>
+      <c r="C122" s="323"/>
+      <c r="D122" s="323"/>
       <c r="E122" s="148">
         <v>4.2000000000000003E-2</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G122" s="45">
         <f>ROUND((E122*D111)/(60*B111),3)</f>
@@ -8531,20 +8501,20 @@
         <f t="shared" si="12"/>
         <v>Pass</v>
       </c>
-      <c r="I122" s="199"/>
+      <c r="I122" s="320"/>
     </row>
     <row r="123" spans="1:15" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="201" t="s">
-        <v>288</v>
-      </c>
-      <c r="B123" s="202"/>
-      <c r="C123" s="202"/>
-      <c r="D123" s="202"/>
+      <c r="A123" s="322" t="s">
+        <v>285</v>
+      </c>
+      <c r="B123" s="323"/>
+      <c r="C123" s="323"/>
+      <c r="D123" s="323"/>
       <c r="E123" s="148">
         <v>2.4E-2</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G123" s="45">
         <f>ROUND((E123*D111)/(60*B111),3)</f>
@@ -8554,26 +8524,26 @@
         <f t="shared" si="12"/>
         <v>Pass</v>
       </c>
-      <c r="I123" s="199"/>
+      <c r="I123" s="320"/>
     </row>
     <row r="124" spans="1:15" ht="14.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A124" s="203" t="s">
-        <v>289</v>
-      </c>
-      <c r="B124" s="204"/>
-      <c r="C124" s="204"/>
-      <c r="D124" s="204"/>
+      <c r="A124" s="324" t="s">
+        <v>286</v>
+      </c>
+      <c r="B124" s="325"/>
+      <c r="C124" s="325"/>
+      <c r="D124" s="325"/>
       <c r="E124" s="150"/>
       <c r="F124" s="151" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G124" s="152" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="H124" s="153" t="s">
-        <v>290</v>
-      </c>
-      <c r="I124" s="200"/>
+        <v>287</v>
+      </c>
+      <c r="I124" s="321"/>
     </row>
     <row r="125" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H125" s="88"/>
@@ -8581,10 +8551,10 @@
     </row>
     <row r="126" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A126" s="158" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C126" s="159" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D126" s="160"/>
       <c r="E126" s="160"/>
@@ -8594,15 +8564,15 @@
       <c r="I126" s="88"/>
     </row>
     <row r="127" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A127" s="180" t="s">
-        <v>293</v>
-      </c>
-      <c r="B127" s="181"/>
-      <c r="C127" s="181"/>
-      <c r="D127" s="181"/>
-      <c r="E127" s="181"/>
-      <c r="F127" s="181"/>
-      <c r="G127" s="182"/>
+      <c r="A127" s="223" t="s">
+        <v>290</v>
+      </c>
+      <c r="B127" s="266"/>
+      <c r="C127" s="266"/>
+      <c r="D127" s="266"/>
+      <c r="E127" s="266"/>
+      <c r="F127" s="266"/>
+      <c r="G127" s="262"/>
       <c r="H127" s="98"/>
       <c r="I127" s="98"/>
       <c r="J127" s="98"/>
@@ -8614,19 +8584,19 @@
     </row>
     <row r="128" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A128" s="99" t="s">
-        <v>294</v>
-      </c>
-      <c r="B128" s="183" t="s">
-        <v>295</v>
-      </c>
-      <c r="C128" s="184"/>
-      <c r="D128" s="184"/>
-      <c r="E128" s="185"/>
+        <v>291</v>
+      </c>
+      <c r="B128" s="194" t="s">
+        <v>292</v>
+      </c>
+      <c r="C128" s="195"/>
+      <c r="D128" s="195"/>
+      <c r="E128" s="196"/>
       <c r="F128" s="162" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="G128" s="163" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H128" s="88"/>
       <c r="I128" s="88"/>
@@ -8642,11 +8612,11 @@
         <v>15</v>
       </c>
       <c r="B129" s="47" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C129" s="105"/>
       <c r="D129" s="164" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E129" s="105"/>
       <c r="F129" s="47" t="e">
@@ -8677,11 +8647,11 @@
         <v>15</v>
       </c>
       <c r="B130" s="102" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C130" s="114"/>
       <c r="D130" s="165" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E130" s="114"/>
       <c r="F130" s="102" t="e">
@@ -8708,15 +8678,15 @@
       <c r="O130" s="98"/>
     </row>
     <row r="131" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A131" s="186" t="s">
-        <v>301</v>
-      </c>
-      <c r="B131" s="176"/>
-      <c r="C131" s="176"/>
-      <c r="D131" s="176"/>
-      <c r="E131" s="176"/>
-      <c r="F131" s="176"/>
-      <c r="G131" s="177"/>
+      <c r="A131" s="336" t="s">
+        <v>298</v>
+      </c>
+      <c r="B131" s="332"/>
+      <c r="C131" s="332"/>
+      <c r="D131" s="332"/>
+      <c r="E131" s="332"/>
+      <c r="F131" s="332"/>
+      <c r="G131" s="333"/>
       <c r="H131" s="88"/>
       <c r="I131" s="88"/>
       <c r="J131" s="88"/>
@@ -8727,15 +8697,15 @@
       <c r="O131" s="98"/>
     </row>
     <row r="132" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="187" t="s">
-        <v>302</v>
-      </c>
-      <c r="B132" s="188"/>
-      <c r="C132" s="188"/>
-      <c r="D132" s="188"/>
-      <c r="E132" s="188"/>
-      <c r="F132" s="188"/>
-      <c r="G132" s="189"/>
+      <c r="A132" s="337" t="s">
+        <v>299</v>
+      </c>
+      <c r="B132" s="338"/>
+      <c r="C132" s="338"/>
+      <c r="D132" s="338"/>
+      <c r="E132" s="338"/>
+      <c r="F132" s="338"/>
+      <c r="G132" s="339"/>
       <c r="H132" s="88"/>
       <c r="I132" s="88"/>
       <c r="J132" s="88"/>
@@ -8746,13 +8716,13 @@
       <c r="O132" s="98"/>
     </row>
     <row r="133" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A133" s="190"/>
-      <c r="B133" s="191"/>
-      <c r="C133" s="191"/>
-      <c r="D133" s="191"/>
-      <c r="E133" s="191"/>
-      <c r="F133" s="191"/>
-      <c r="G133" s="192"/>
+      <c r="A133" s="340"/>
+      <c r="B133" s="341"/>
+      <c r="C133" s="341"/>
+      <c r="D133" s="341"/>
+      <c r="E133" s="341"/>
+      <c r="F133" s="341"/>
+      <c r="G133" s="342"/>
       <c r="H133" s="98"/>
       <c r="I133" s="98"/>
       <c r="J133" s="98"/>
@@ -8774,7 +8744,7 @@
     </row>
     <row r="135" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A135" s="166" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B135" s="129"/>
       <c r="C135" s="129"/>
@@ -8782,7 +8752,7 @@
         <v>0</v>
       </c>
       <c r="E135" s="168" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F135" s="169" t="str">
         <f>IF(D135&lt;=5,"Pass","Fail")</f>
@@ -8818,7 +8788,7 @@
     </row>
     <row r="138" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A138" s="44" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H138" s="98"/>
       <c r="I138" s="98"/>
@@ -8859,7 +8829,7 @@
       <c r="O139" s="98"/>
     </row>
     <row r="140" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A140" s="193" t="s">
+      <c r="A140" s="343" t="s">
         <v>2</v>
       </c>
       <c r="B140" s="20">
@@ -8890,7 +8860,7 @@
       <c r="O140" s="98"/>
     </row>
     <row r="141" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A141" s="194"/>
+      <c r="A141" s="312"/>
       <c r="B141" s="20">
         <f>B140-B140</f>
         <v>0</v>
@@ -8926,8 +8896,8 @@
     </row>
     <row r="142" spans="1:15" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="96"/>
-      <c r="B142" s="195" t="s">
-        <v>306</v>
+      <c r="B142" s="344" t="s">
+        <v>303</v>
       </c>
       <c r="C142" s="173">
         <f>C139-C141</f>
@@ -8960,7 +8930,7 @@
     </row>
     <row r="143" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="96"/>
-      <c r="B143" s="195"/>
+      <c r="B143" s="344"/>
       <c r="C143" s="20" t="str">
         <f t="shared" ref="C143:E143" si="14">IF(C142&gt;1,"Fail","Pass")</f>
         <v>Pass</v>
@@ -8991,26 +8961,26 @@
       <c r="O143" s="98"/>
     </row>
     <row r="144" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A144" s="175" t="s">
-        <v>307</v>
-      </c>
-      <c r="B144" s="176"/>
-      <c r="C144" s="176"/>
-      <c r="D144" s="176"/>
-      <c r="E144" s="176"/>
-      <c r="F144" s="176"/>
-      <c r="G144" s="177"/>
+      <c r="A144" s="331" t="s">
+        <v>304</v>
+      </c>
+      <c r="B144" s="332"/>
+      <c r="C144" s="332"/>
+      <c r="D144" s="332"/>
+      <c r="E144" s="332"/>
+      <c r="F144" s="332"/>
+      <c r="G144" s="333"/>
     </row>
     <row r="145" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A145" s="175" t="s">
-        <v>308</v>
-      </c>
-      <c r="B145" s="178"/>
-      <c r="C145" s="178"/>
-      <c r="D145" s="178"/>
-      <c r="E145" s="178"/>
-      <c r="F145" s="178"/>
-      <c r="G145" s="179"/>
+      <c r="A145" s="331" t="s">
+        <v>305</v>
+      </c>
+      <c r="B145" s="334"/>
+      <c r="C145" s="334"/>
+      <c r="D145" s="334"/>
+      <c r="E145" s="334"/>
+      <c r="F145" s="334"/>
+      <c r="G145" s="335"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -9026,107 +8996,26 @@
     <protectedRange sqref="A126" name="Range10"/>
   </protectedRanges>
   <mergeCells count="136">
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="P11:X11"/>
-    <mergeCell ref="P12:P13"/>
-    <mergeCell ref="Q12:S12"/>
-    <mergeCell ref="T12:T13"/>
-    <mergeCell ref="U12:U13"/>
-    <mergeCell ref="V12:V13"/>
-    <mergeCell ref="X12:X13"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B10:I10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="P25:U25"/>
-    <mergeCell ref="P27:R27"/>
-    <mergeCell ref="P18:V18"/>
-    <mergeCell ref="P19:V19"/>
-    <mergeCell ref="P20:U20"/>
-    <mergeCell ref="P21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="H65:I65"/>
-    <mergeCell ref="P41:Y41"/>
-    <mergeCell ref="P43:Q43"/>
-    <mergeCell ref="P45:S47"/>
-    <mergeCell ref="A57:I57"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="Q28:S28"/>
-    <mergeCell ref="U29:U32"/>
-    <mergeCell ref="X29:X32"/>
-    <mergeCell ref="P33:X33"/>
-    <mergeCell ref="P35:Y35"/>
-    <mergeCell ref="Q36:U36"/>
-    <mergeCell ref="H66:I66"/>
-    <mergeCell ref="H69:I69"/>
-    <mergeCell ref="P69:Q69"/>
-    <mergeCell ref="R69:S69"/>
-    <mergeCell ref="H70:I70"/>
-    <mergeCell ref="P70:Q70"/>
-    <mergeCell ref="R70:S70"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="H62:I62"/>
-    <mergeCell ref="H63:I63"/>
-    <mergeCell ref="H64:I64"/>
-    <mergeCell ref="H73:I73"/>
-    <mergeCell ref="P73:Q73"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="H74:I74"/>
-    <mergeCell ref="P74:Q74"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="H71:I71"/>
-    <mergeCell ref="P71:Q71"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="H72:I72"/>
-    <mergeCell ref="P72:Q72"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="D82:D86"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="H75:I75"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="A77:I77"/>
-    <mergeCell ref="A80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="H81:I81"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="D96:E96"/>
-    <mergeCell ref="A97:B97"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="A98:E99"/>
-    <mergeCell ref="A101:J101"/>
-    <mergeCell ref="A87:F88"/>
-    <mergeCell ref="C90:E90"/>
-    <mergeCell ref="D91:E91"/>
-    <mergeCell ref="A92:B92"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A144:G144"/>
+    <mergeCell ref="A145:G145"/>
+    <mergeCell ref="A127:G127"/>
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="A131:G131"/>
+    <mergeCell ref="A132:G133"/>
+    <mergeCell ref="A140:A141"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="A120:D120"/>
+    <mergeCell ref="I120:I124"/>
+    <mergeCell ref="A121:D121"/>
+    <mergeCell ref="A122:D122"/>
+    <mergeCell ref="A123:D123"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="I115:I119"/>
+    <mergeCell ref="A116:D116"/>
+    <mergeCell ref="A117:D117"/>
+    <mergeCell ref="A118:D118"/>
+    <mergeCell ref="A119:D119"/>
     <mergeCell ref="A106:L106"/>
     <mergeCell ref="A113:D114"/>
     <mergeCell ref="E113:F114"/>
@@ -9142,26 +9031,107 @@
     <mergeCell ref="G105:H105"/>
     <mergeCell ref="I105:J105"/>
     <mergeCell ref="K105:L105"/>
-    <mergeCell ref="I120:I124"/>
-    <mergeCell ref="A121:D121"/>
-    <mergeCell ref="A122:D122"/>
-    <mergeCell ref="A123:D123"/>
-    <mergeCell ref="A124:D124"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="I115:I119"/>
-    <mergeCell ref="A116:D116"/>
-    <mergeCell ref="A117:D117"/>
-    <mergeCell ref="A118:D118"/>
-    <mergeCell ref="A119:D119"/>
-    <mergeCell ref="A144:G144"/>
-    <mergeCell ref="A145:G145"/>
-    <mergeCell ref="A127:G127"/>
-    <mergeCell ref="B128:E128"/>
-    <mergeCell ref="A131:G131"/>
-    <mergeCell ref="A132:G133"/>
-    <mergeCell ref="A140:A141"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="A120:D120"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="D96:E96"/>
+    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="A98:E99"/>
+    <mergeCell ref="A101:J101"/>
+    <mergeCell ref="A87:F88"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="D91:E91"/>
+    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="D82:D86"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="H75:I75"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="A80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="H81:I81"/>
+    <mergeCell ref="H73:I73"/>
+    <mergeCell ref="P73:Q73"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="H74:I74"/>
+    <mergeCell ref="P74:Q74"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="H71:I71"/>
+    <mergeCell ref="P71:Q71"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="H72:I72"/>
+    <mergeCell ref="P72:Q72"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="H66:I66"/>
+    <mergeCell ref="H69:I69"/>
+    <mergeCell ref="P69:Q69"/>
+    <mergeCell ref="R69:S69"/>
+    <mergeCell ref="H70:I70"/>
+    <mergeCell ref="P70:Q70"/>
+    <mergeCell ref="R70:S70"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="H62:I62"/>
+    <mergeCell ref="H63:I63"/>
+    <mergeCell ref="H64:I64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="H65:I65"/>
+    <mergeCell ref="P41:Y41"/>
+    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="P45:S47"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="Q28:S28"/>
+    <mergeCell ref="U29:U32"/>
+    <mergeCell ref="X29:X32"/>
+    <mergeCell ref="P33:X33"/>
+    <mergeCell ref="P35:Y35"/>
+    <mergeCell ref="Q36:U36"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="P25:U25"/>
+    <mergeCell ref="P27:R27"/>
+    <mergeCell ref="P18:V18"/>
+    <mergeCell ref="P19:V19"/>
+    <mergeCell ref="P20:U20"/>
+    <mergeCell ref="P21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="P11:X11"/>
+    <mergeCell ref="P12:P13"/>
+    <mergeCell ref="Q12:S12"/>
+    <mergeCell ref="T12:T13"/>
+    <mergeCell ref="U12:U13"/>
+    <mergeCell ref="V12:V13"/>
+    <mergeCell ref="X12:X13"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="C142:G142">
     <cfRule type="cellIs" dxfId="40" priority="6" operator="greaterThan">

</xml_diff>

<commit_message>
Enhance CT template generation by refactoring file paths to use dynamic directory resolution, adding a new Dental CBCT template for input-only data, and updating existing CSV templates for improved structure and clarity. Adjusted tolerance handling in BMD report components and optimized data loading logic for better performance.
</commit_message>
<xml_diff>
--- a/public/templates/CTScan_SingleTube_Sample.xlsx
+++ b/public/templates/CTScan_SingleTube_Sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECTS\anteso\anteso-frontend\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PRAJWALA\anteso\anteso-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6ED6AA3-2B6F-4A58-87D1-12226F984847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E72E0679-3BF4-4202-8C44-14D26C8B090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,17 @@
     <sheet name="raw data" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -991,7 +1002,7 @@
     <t>Note : Where I is + value &amp; S is - value &amp; vise versa if applicable</t>
   </si>
   <si>
-    <t xml:space="preserve"> mA 10</t>
+    <t xml:space="preserve"> @mA 10</t>
   </si>
 </sst>
 </file>
@@ -2465,6 +2476,474 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2480,24 +2959,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2522,9 +2983,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2533,453 +2991,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4989,38 +5000,38 @@
       <c r="A1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="342" t="s">
+      <c r="B1" s="175" t="s">
         <v>139</v>
       </c>
-      <c r="C1" s="342"/>
-      <c r="D1" s="342"/>
-      <c r="E1" s="342"/>
-      <c r="F1" s="342"/>
-      <c r="G1" s="342"/>
-      <c r="H1" s="342"/>
-      <c r="I1" s="342"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="346"/>
-      <c r="L1" s="346"/>
-      <c r="M1" s="346"/>
-      <c r="N1" s="222"/>
-      <c r="O1" s="222"/>
+      <c r="K1" s="177"/>
+      <c r="L1" s="177"/>
+      <c r="M1" s="177"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
       <c r="P1" s="3"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="342" t="s">
+      <c r="B2" s="175" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="342"/>
-      <c r="D2" s="342"/>
-      <c r="E2" s="342"/>
-      <c r="F2" s="342"/>
-      <c r="G2" s="342"/>
-      <c r="H2" s="342"/>
-      <c r="I2" s="342"/>
+      <c r="C2" s="175"/>
+      <c r="D2" s="175"/>
+      <c r="E2" s="175"/>
+      <c r="F2" s="175"/>
+      <c r="G2" s="175"/>
+      <c r="H2" s="175"/>
+      <c r="I2" s="175"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -5030,16 +5041,16 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="342" t="s">
+      <c r="B3" s="175" t="s">
         <v>142</v>
       </c>
-      <c r="C3" s="342"/>
-      <c r="D3" s="342"/>
-      <c r="E3" s="342"/>
-      <c r="F3" s="342"/>
-      <c r="G3" s="342"/>
-      <c r="H3" s="342"/>
-      <c r="I3" s="342"/>
+      <c r="C3" s="175"/>
+      <c r="D3" s="175"/>
+      <c r="E3" s="175"/>
+      <c r="F3" s="175"/>
+      <c r="G3" s="175"/>
+      <c r="H3" s="175"/>
+      <c r="I3" s="175"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -5051,14 +5062,14 @@
       <c r="A4" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="B4" s="342"/>
-      <c r="C4" s="342"/>
-      <c r="D4" s="342"/>
-      <c r="E4" s="342"/>
-      <c r="F4" s="342"/>
-      <c r="G4" s="342"/>
-      <c r="H4" s="342"/>
-      <c r="I4" s="342"/>
+      <c r="B4" s="175"/>
+      <c r="C4" s="175"/>
+      <c r="D4" s="175"/>
+      <c r="E4" s="175"/>
+      <c r="F4" s="175"/>
+      <c r="G4" s="175"/>
+      <c r="H4" s="175"/>
+      <c r="I4" s="175"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -5070,20 +5081,20 @@
       <c r="A5" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="342" t="s">
+      <c r="B5" s="175" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="342"/>
-      <c r="D5" s="342"/>
-      <c r="E5" s="342"/>
+      <c r="C5" s="175"/>
+      <c r="D5" s="175"/>
+      <c r="E5" s="175"/>
       <c r="F5" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="G5" s="345">
+      <c r="G5" s="176">
         <v>22.7</v>
       </c>
-      <c r="H5" s="345"/>
-      <c r="I5" s="345"/>
+      <c r="H5" s="176"/>
+      <c r="I5" s="176"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -5095,20 +5106,20 @@
       <c r="A6" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B6" s="342" t="s">
+      <c r="B6" s="175" t="s">
         <v>148</v>
       </c>
-      <c r="C6" s="342"/>
-      <c r="D6" s="342"/>
-      <c r="E6" s="342"/>
+      <c r="C6" s="175"/>
+      <c r="D6" s="175"/>
+      <c r="E6" s="175"/>
       <c r="F6" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G6" s="345">
+      <c r="G6" s="176">
         <v>50.2</v>
       </c>
-      <c r="H6" s="345"/>
-      <c r="I6" s="345"/>
+      <c r="H6" s="176"/>
+      <c r="I6" s="176"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -5120,20 +5131,20 @@
       <c r="A7" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="342" t="s">
+      <c r="B7" s="175" t="s">
         <v>151</v>
       </c>
-      <c r="C7" s="342"/>
-      <c r="D7" s="342"/>
-      <c r="E7" s="342"/>
+      <c r="C7" s="175"/>
+      <c r="D7" s="175"/>
+      <c r="E7" s="175"/>
       <c r="F7" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="342" t="s">
+      <c r="G7" s="175" t="s">
         <v>152</v>
       </c>
-      <c r="H7" s="342"/>
-      <c r="I7" s="342"/>
+      <c r="H7" s="175"/>
+      <c r="I7" s="175"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -5144,16 +5155,16 @@
       <c r="A8" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="341">
+      <c r="B8" s="191">
         <v>46066</v>
       </c>
-      <c r="C8" s="342"/>
-      <c r="D8" s="342"/>
-      <c r="E8" s="342"/>
+      <c r="C8" s="175"/>
+      <c r="D8" s="175"/>
+      <c r="E8" s="175"/>
       <c r="F8" s="4"/>
-      <c r="G8" s="342"/>
-      <c r="H8" s="342"/>
-      <c r="I8" s="342"/>
+      <c r="G8" s="175"/>
+      <c r="H8" s="175"/>
+      <c r="I8" s="175"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -5162,14 +5173,14 @@
     </row>
     <row r="9" spans="1:27" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="336"/>
-      <c r="C9" s="336"/>
-      <c r="D9" s="336"/>
-      <c r="E9" s="336"/>
+      <c r="B9" s="184"/>
+      <c r="C9" s="184"/>
+      <c r="D9" s="184"/>
+      <c r="E9" s="184"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="336"/>
-      <c r="H9" s="336"/>
-      <c r="I9" s="336"/>
+      <c r="G9" s="184"/>
+      <c r="H9" s="184"/>
+      <c r="I9" s="184"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -5180,16 +5191,16 @@
       <c r="A10" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="B10" s="343" t="s">
+      <c r="B10" s="192" t="s">
         <v>155</v>
       </c>
-      <c r="C10" s="343"/>
-      <c r="D10" s="343"/>
-      <c r="E10" s="343"/>
-      <c r="F10" s="343"/>
-      <c r="G10" s="343"/>
-      <c r="H10" s="343"/>
-      <c r="I10" s="344"/>
+      <c r="C10" s="192"/>
+      <c r="D10" s="192"/>
+      <c r="E10" s="192"/>
+      <c r="F10" s="192"/>
+      <c r="G10" s="192"/>
+      <c r="H10" s="192"/>
+      <c r="I10" s="193"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -5197,35 +5208,35 @@
       <c r="N10" s="2"/>
     </row>
     <row r="11" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="183" t="s">
+      <c r="A11" s="194" t="s">
         <v>156</v>
       </c>
-      <c r="B11" s="184"/>
-      <c r="C11" s="185"/>
-      <c r="D11" s="184" t="s">
+      <c r="B11" s="195"/>
+      <c r="C11" s="196"/>
+      <c r="D11" s="195" t="s">
         <v>157</v>
       </c>
-      <c r="E11" s="184"/>
-      <c r="F11" s="184"/>
-      <c r="G11" s="184"/>
-      <c r="H11" s="184"/>
-      <c r="I11" s="185"/>
+      <c r="E11" s="195"/>
+      <c r="F11" s="195"/>
+      <c r="G11" s="195"/>
+      <c r="H11" s="195"/>
+      <c r="I11" s="196"/>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="9"/>
-      <c r="P11" s="331" t="s">
+      <c r="P11" s="179" t="s">
         <v>158</v>
       </c>
-      <c r="Q11" s="332"/>
-      <c r="R11" s="332"/>
-      <c r="S11" s="332"/>
-      <c r="T11" s="332"/>
-      <c r="U11" s="332"/>
-      <c r="V11" s="332"/>
-      <c r="W11" s="332"/>
-      <c r="X11" s="333"/>
+      <c r="Q11" s="180"/>
+      <c r="R11" s="180"/>
+      <c r="S11" s="180"/>
+      <c r="T11" s="180"/>
+      <c r="U11" s="180"/>
+      <c r="V11" s="180"/>
+      <c r="W11" s="180"/>
+      <c r="X11" s="181"/>
     </row>
     <row r="12" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
@@ -5264,23 +5275,23 @@
       <c r="N12" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="P12" s="334" t="s">
+      <c r="P12" s="182" t="s">
         <v>166</v>
       </c>
-      <c r="Q12" s="336" t="s">
+      <c r="Q12" s="184" t="s">
         <v>167</v>
       </c>
-      <c r="R12" s="336"/>
-      <c r="S12" s="336"/>
-      <c r="T12" s="337" t="s">
+      <c r="R12" s="184"/>
+      <c r="S12" s="184"/>
+      <c r="T12" s="185" t="s">
         <v>168</v>
       </c>
-      <c r="U12" s="305" t="s">
+      <c r="U12" s="187" t="s">
         <v>169</v>
       </c>
-      <c r="V12" s="337"/>
+      <c r="V12" s="185"/>
       <c r="W12" s="5"/>
-      <c r="X12" s="339" t="s">
+      <c r="X12" s="189" t="s">
         <v>170</v>
       </c>
     </row>
@@ -5320,7 +5331,7 @@
         <f>ROUND(F13,4)</f>
         <v>0.53200000000000003</v>
       </c>
-      <c r="P13" s="335"/>
+      <c r="P13" s="183"/>
       <c r="Q13" s="17">
         <f>B14</f>
         <v>10</v>
@@ -5333,11 +5344,11 @@
         <f>B22</f>
         <v>350</v>
       </c>
-      <c r="T13" s="338"/>
-      <c r="U13" s="216"/>
-      <c r="V13" s="338"/>
+      <c r="T13" s="186"/>
+      <c r="U13" s="188"/>
+      <c r="V13" s="186"/>
       <c r="W13" s="19"/>
-      <c r="X13" s="340"/>
+      <c r="X13" s="190"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="20">
@@ -5649,15 +5660,15 @@
         <f t="shared" si="0"/>
         <v>5.2999000000000001</v>
       </c>
-      <c r="P18" s="325" t="s">
+      <c r="P18" s="206" t="s">
         <v>174</v>
       </c>
-      <c r="Q18" s="326"/>
-      <c r="R18" s="326"/>
-      <c r="S18" s="326"/>
-      <c r="T18" s="326"/>
-      <c r="U18" s="326"/>
-      <c r="V18" s="327"/>
+      <c r="Q18" s="207"/>
+      <c r="R18" s="207"/>
+      <c r="S18" s="207"/>
+      <c r="T18" s="207"/>
+      <c r="U18" s="207"/>
+      <c r="V18" s="208"/>
       <c r="W18" s="40"/>
       <c r="X18" s="41"/>
     </row>
@@ -5697,13 +5708,13 @@
         <f t="shared" si="0"/>
         <v>5.3005000000000004</v>
       </c>
-      <c r="P19" s="289"/>
-      <c r="Q19" s="289"/>
-      <c r="R19" s="289"/>
-      <c r="S19" s="289"/>
-      <c r="T19" s="289"/>
-      <c r="U19" s="289"/>
-      <c r="V19" s="289"/>
+      <c r="P19" s="209"/>
+      <c r="Q19" s="209"/>
+      <c r="R19" s="209"/>
+      <c r="S19" s="209"/>
+      <c r="T19" s="209"/>
+      <c r="U19" s="209"/>
+      <c r="V19" s="209"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20" s="20">
@@ -5741,14 +5752,14 @@
         <f t="shared" si="0"/>
         <v>5.3002000000000002</v>
       </c>
-      <c r="P20" s="310" t="s">
+      <c r="P20" s="210" t="s">
         <v>175</v>
       </c>
-      <c r="Q20" s="311"/>
-      <c r="R20" s="311"/>
-      <c r="S20" s="311"/>
-      <c r="T20" s="311"/>
-      <c r="U20" s="313"/>
+      <c r="Q20" s="211"/>
+      <c r="R20" s="211"/>
+      <c r="S20" s="211"/>
+      <c r="T20" s="211"/>
+      <c r="U20" s="212"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="20">
@@ -5786,14 +5797,14 @@
         <f t="shared" si="0"/>
         <v>5.2969999999999997</v>
       </c>
-      <c r="P21" s="328" t="s">
+      <c r="P21" s="213" t="s">
         <v>176</v>
       </c>
-      <c r="Q21" s="329"/>
-      <c r="R21" s="330" t="s">
+      <c r="Q21" s="214"/>
+      <c r="R21" s="215" t="s">
         <v>177</v>
       </c>
-      <c r="S21" s="329"/>
+      <c r="S21" s="214"/>
       <c r="T21" s="14" t="s">
         <v>178</v>
       </c>
@@ -5840,16 +5851,16 @@
         <f t="shared" si="0"/>
         <v>18.497399999999999</v>
       </c>
-      <c r="P22" s="316">
+      <c r="P22" s="197">
         <f>C14</f>
         <v>1</v>
       </c>
-      <c r="Q22" s="317"/>
-      <c r="R22" s="318">
+      <c r="Q22" s="198"/>
+      <c r="R22" s="199">
         <f>ROUND(E14/1000,4)</f>
         <v>1.0092000000000001</v>
       </c>
-      <c r="S22" s="318"/>
+      <c r="S22" s="199"/>
       <c r="T22" s="45">
         <f>ROUND(ABS(((R22-P22)/P22*100)),2)</f>
         <v>0.92</v>
@@ -5895,16 +5906,16 @@
         <f t="shared" si="0"/>
         <v>0.94920000000000004</v>
       </c>
-      <c r="P23" s="316">
+      <c r="P23" s="197">
         <f>C15</f>
         <v>2</v>
       </c>
-      <c r="Q23" s="317"/>
-      <c r="R23" s="318">
+      <c r="Q23" s="198"/>
+      <c r="R23" s="199">
         <f>ROUND(E15/1000,4)</f>
         <v>2.0093999999999999</v>
       </c>
-      <c r="S23" s="318"/>
+      <c r="S23" s="199"/>
       <c r="T23" s="45">
         <f>ROUND(ABS(((R23-P23)/P23*100)),2)</f>
         <v>0.47</v>
@@ -5950,16 +5961,16 @@
         <f t="shared" si="0"/>
         <v>9.4794</v>
       </c>
-      <c r="P24" s="316">
+      <c r="P24" s="197">
         <f>C16</f>
         <v>3</v>
       </c>
-      <c r="Q24" s="317"/>
-      <c r="R24" s="318">
+      <c r="Q24" s="198"/>
+      <c r="R24" s="199">
         <f>ROUND(E16/1000,4)</f>
         <v>3.0081000000000002</v>
       </c>
-      <c r="S24" s="318"/>
+      <c r="S24" s="199"/>
       <c r="T24" s="45">
         <f>ROUND(ABS(((R24-P24)/P24*100)),2)</f>
         <v>0.27</v>
@@ -6005,14 +6016,14 @@
         <f t="shared" si="0"/>
         <v>9.4793000000000003</v>
       </c>
-      <c r="P25" s="319" t="s">
+      <c r="P25" s="200" t="s">
         <v>180</v>
       </c>
-      <c r="Q25" s="320"/>
-      <c r="R25" s="320"/>
-      <c r="S25" s="320"/>
-      <c r="T25" s="320"/>
-      <c r="U25" s="321"/>
+      <c r="Q25" s="201"/>
+      <c r="R25" s="201"/>
+      <c r="S25" s="201"/>
+      <c r="T25" s="201"/>
+      <c r="U25" s="202"/>
     </row>
     <row r="26" spans="1:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="20">
@@ -6087,11 +6098,11 @@
         <f t="shared" si="0"/>
         <v>9.4781999999999993</v>
       </c>
-      <c r="P27" s="322" t="s">
+      <c r="P27" s="203" t="s">
         <v>181</v>
       </c>
-      <c r="Q27" s="323"/>
-      <c r="R27" s="324"/>
+      <c r="Q27" s="204"/>
+      <c r="R27" s="205"/>
       <c r="S27" s="47" t="s">
         <v>159</v>
       </c>
@@ -6148,11 +6159,11 @@
       <c r="P28" s="30" t="s">
         <v>183</v>
       </c>
-      <c r="Q28" s="305" t="s">
+      <c r="Q28" s="187" t="s">
         <v>184</v>
       </c>
-      <c r="R28" s="305"/>
-      <c r="S28" s="305"/>
+      <c r="R28" s="187"/>
+      <c r="S28" s="187"/>
       <c r="T28" s="14" t="s">
         <v>185</v>
       </c>
@@ -6224,13 +6235,13 @@
         <f>ROUND((AVERAGE(Q29:S29)/(P29*X27)),4)</f>
         <v>0.1457</v>
       </c>
-      <c r="U29" s="306">
+      <c r="U29" s="237">
         <f>ROUND((MAX(T29:T32)-MIN(T29:T32))/(MAX(T29:T32)+MIN(T29:T32)),4)</f>
         <v>1.4E-3</v>
       </c>
       <c r="V29" s="13"/>
       <c r="W29" s="5"/>
-      <c r="X29" s="308" t="str">
+      <c r="X29" s="239" t="str">
         <f>IF(U29&lt;0.1,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
@@ -6291,10 +6302,10 @@
         <f>ROUND((AVERAGE(Q30:S30)/(P30*X27)),4)</f>
         <v>0.14530000000000001</v>
       </c>
-      <c r="U30" s="306"/>
+      <c r="U30" s="237"/>
       <c r="V30" s="13"/>
       <c r="W30" s="5"/>
-      <c r="X30" s="308"/>
+      <c r="X30" s="239"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A31" s="20">
@@ -6352,10 +6363,10 @@
         <f>ROUND((AVERAGE(Q31:S31)/(P31*X27)),4)</f>
         <v>0.14549999999999999</v>
       </c>
-      <c r="U31" s="306"/>
+      <c r="U31" s="237"/>
       <c r="V31" s="13"/>
       <c r="W31" s="5"/>
-      <c r="X31" s="308"/>
+      <c r="X31" s="239"/>
     </row>
     <row r="32" spans="1:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="20">
@@ -6413,10 +6424,10 @@
         <f>ROUND((AVERAGE(Q32:S32)/(P32*X27)),4)</f>
         <v>0.1454</v>
       </c>
-      <c r="U32" s="307"/>
+      <c r="U32" s="238"/>
       <c r="V32" s="18"/>
       <c r="W32" s="19"/>
-      <c r="X32" s="309"/>
+      <c r="X32" s="240"/>
     </row>
     <row r="33" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="20">
@@ -6454,17 +6465,17 @@
         <f t="shared" si="0"/>
         <v>7.2878999999999996</v>
       </c>
-      <c r="P33" s="210" t="s">
+      <c r="P33" s="220" t="s">
         <v>187</v>
       </c>
-      <c r="Q33" s="211"/>
-      <c r="R33" s="211"/>
-      <c r="S33" s="211"/>
-      <c r="T33" s="211"/>
-      <c r="U33" s="211"/>
-      <c r="V33" s="211"/>
-      <c r="W33" s="211"/>
-      <c r="X33" s="212"/>
+      <c r="Q33" s="221"/>
+      <c r="R33" s="221"/>
+      <c r="S33" s="221"/>
+      <c r="T33" s="221"/>
+      <c r="U33" s="221"/>
+      <c r="V33" s="221"/>
+      <c r="W33" s="221"/>
+      <c r="X33" s="222"/>
     </row>
     <row r="34" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="20">
@@ -6539,18 +6550,18 @@
         <f t="shared" si="0"/>
         <v>14.5259</v>
       </c>
-      <c r="P35" s="310" t="s">
+      <c r="P35" s="210" t="s">
         <v>188</v>
       </c>
-      <c r="Q35" s="311"/>
-      <c r="R35" s="311"/>
-      <c r="S35" s="311"/>
-      <c r="T35" s="311"/>
-      <c r="U35" s="311"/>
-      <c r="V35" s="312"/>
-      <c r="W35" s="312"/>
-      <c r="X35" s="312"/>
-      <c r="Y35" s="313"/>
+      <c r="Q35" s="211"/>
+      <c r="R35" s="211"/>
+      <c r="S35" s="211"/>
+      <c r="T35" s="211"/>
+      <c r="U35" s="211"/>
+      <c r="V35" s="241"/>
+      <c r="W35" s="241"/>
+      <c r="X35" s="241"/>
+      <c r="Y35" s="212"/>
     </row>
     <row r="36" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="20">
@@ -6591,13 +6602,13 @@
       <c r="P36" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="Q36" s="314" t="s">
+      <c r="Q36" s="242" t="s">
         <v>184</v>
       </c>
-      <c r="R36" s="314"/>
-      <c r="S36" s="314"/>
-      <c r="T36" s="314"/>
-      <c r="U36" s="315"/>
+      <c r="R36" s="242"/>
+      <c r="S36" s="242"/>
+      <c r="T36" s="242"/>
+      <c r="U36" s="243"/>
       <c r="V36" s="18" t="s">
         <v>189</v>
       </c>
@@ -6955,18 +6966,18 @@
         <f t="shared" si="0"/>
         <v>29.098600000000001</v>
       </c>
-      <c r="P41" s="210" t="s">
+      <c r="P41" s="220" t="s">
         <v>191</v>
       </c>
-      <c r="Q41" s="211"/>
-      <c r="R41" s="211"/>
-      <c r="S41" s="211"/>
-      <c r="T41" s="211"/>
-      <c r="U41" s="211"/>
-      <c r="V41" s="211"/>
-      <c r="W41" s="211"/>
-      <c r="X41" s="211"/>
-      <c r="Y41" s="212"/>
+      <c r="Q41" s="221"/>
+      <c r="R41" s="221"/>
+      <c r="S41" s="221"/>
+      <c r="T41" s="221"/>
+      <c r="U41" s="221"/>
+      <c r="V41" s="221"/>
+      <c r="W41" s="221"/>
+      <c r="X41" s="221"/>
+      <c r="Y41" s="222"/>
     </row>
     <row r="42" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="20">
@@ -7044,10 +7055,10 @@
         <f t="shared" si="0"/>
         <v>50.876800000000003</v>
       </c>
-      <c r="P43" s="180" t="s">
+      <c r="P43" s="223" t="s">
         <v>192</v>
       </c>
-      <c r="Q43" s="296"/>
+      <c r="Q43" s="224"/>
       <c r="R43" s="72" t="s">
         <v>164</v>
       </c>
@@ -7143,12 +7154,12 @@
         <f t="shared" si="0"/>
         <v>2.0246</v>
       </c>
-      <c r="P45" s="297" t="s">
+      <c r="P45" s="225" t="s">
         <v>193</v>
       </c>
-      <c r="Q45" s="298"/>
-      <c r="R45" s="298"/>
-      <c r="S45" s="299"/>
+      <c r="Q45" s="226"/>
+      <c r="R45" s="226"/>
+      <c r="S45" s="227"/>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A46" s="20">
@@ -7186,10 +7197,10 @@
         <f t="shared" si="0"/>
         <v>20.186800000000002</v>
       </c>
-      <c r="P46" s="297"/>
-      <c r="Q46" s="298"/>
-      <c r="R46" s="298"/>
-      <c r="S46" s="299"/>
+      <c r="P46" s="225"/>
+      <c r="Q46" s="226"/>
+      <c r="R46" s="226"/>
+      <c r="S46" s="227"/>
     </row>
     <row r="47" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="20">
@@ -7227,9 +7238,9 @@
         <f t="shared" si="0"/>
         <v>20.193899999999999</v>
       </c>
-      <c r="P47" s="229"/>
-      <c r="Q47" s="300"/>
-      <c r="R47" s="300"/>
+      <c r="P47" s="228"/>
+      <c r="Q47" s="229"/>
+      <c r="R47" s="229"/>
       <c r="S47" s="230"/>
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.3">
@@ -7444,17 +7455,17 @@
       <c r="J56" s="80"/>
     </row>
     <row r="57" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="301" t="s">
+      <c r="A57" s="231" t="s">
         <v>194</v>
       </c>
-      <c r="B57" s="302"/>
-      <c r="C57" s="302"/>
-      <c r="D57" s="302"/>
-      <c r="E57" s="302"/>
-      <c r="F57" s="302"/>
-      <c r="G57" s="302"/>
-      <c r="H57" s="302"/>
-      <c r="I57" s="303"/>
+      <c r="B57" s="232"/>
+      <c r="C57" s="232"/>
+      <c r="D57" s="232"/>
+      <c r="E57" s="232"/>
+      <c r="F57" s="232"/>
+      <c r="G57" s="232"/>
+      <c r="H57" s="232"/>
+      <c r="I57" s="233"/>
       <c r="J57" s="80"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
@@ -7496,10 +7507,10 @@
       <c r="G59" s="87" t="s">
         <v>204</v>
       </c>
-      <c r="H59" s="291" t="s">
+      <c r="H59" s="234" t="s">
         <v>205</v>
       </c>
-      <c r="I59" s="292"/>
+      <c r="I59" s="235"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="86"/>
@@ -7518,30 +7529,30 @@
       <c r="F60" t="s">
         <v>60</v>
       </c>
-      <c r="H60" s="304">
+      <c r="H60" s="236">
         <v>18.12</v>
       </c>
-      <c r="I60" s="304"/>
+      <c r="I60" s="236"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="86"/>
       <c r="F61" t="s">
         <v>62</v>
       </c>
-      <c r="H61" s="287">
+      <c r="H61" s="248">
         <v>19.98</v>
       </c>
-      <c r="I61" s="287"/>
+      <c r="I61" s="248"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="86"/>
       <c r="F62" t="s">
         <v>65</v>
       </c>
-      <c r="H62" s="287">
+      <c r="H62" s="248">
         <v>18.7</v>
       </c>
-      <c r="I62" s="287"/>
+      <c r="I62" s="248"/>
       <c r="J62" s="88"/>
       <c r="K62" s="88"/>
     </row>
@@ -7550,10 +7561,10 @@
       <c r="F63" t="s">
         <v>207</v>
       </c>
-      <c r="H63" s="287">
+      <c r="H63" s="248">
         <v>17.62</v>
       </c>
-      <c r="I63" s="287"/>
+      <c r="I63" s="248"/>
       <c r="J63" s="88"/>
       <c r="K63" s="88"/>
     </row>
@@ -7562,27 +7573,27 @@
       <c r="F64" t="s">
         <v>208</v>
       </c>
-      <c r="H64" s="290">
+      <c r="H64" s="249">
         <v>18.79</v>
       </c>
-      <c r="I64" s="290"/>
+      <c r="I64" s="249"/>
       <c r="J64" s="88"/>
       <c r="K64" s="88"/>
     </row>
     <row r="65" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="86"/>
-      <c r="B65" s="277" t="s">
+      <c r="B65" s="216" t="s">
         <v>209</v>
       </c>
-      <c r="C65" s="278"/>
+      <c r="C65" s="217"/>
       <c r="D65" s="91">
         <v>18.05</v>
       </c>
-      <c r="H65" s="294">
+      <c r="H65" s="218">
         <f>(H60/3)+(2/3*J65)</f>
         <v>18.555</v>
       </c>
-      <c r="I65" s="295"/>
+      <c r="I65" s="219"/>
       <c r="J65" s="92">
         <f>AVERAGE(H61:I64)</f>
         <v>18.772500000000001</v>
@@ -7597,11 +7608,11 @@
       <c r="G66" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H66" s="242" t="str">
+      <c r="H66" s="244" t="str">
         <f>IF(K65&lt;20,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I66" s="244"/>
+      <c r="I66" s="245"/>
       <c r="J66" s="88"/>
       <c r="K66" s="88"/>
       <c r="P66" s="2"/>
@@ -7662,14 +7673,14 @@
       <c r="G69" s="87" t="s">
         <v>204</v>
       </c>
-      <c r="H69" s="291" t="s">
+      <c r="H69" s="234" t="s">
         <v>205</v>
       </c>
-      <c r="I69" s="292"/>
-      <c r="P69" s="288"/>
-      <c r="Q69" s="288"/>
-      <c r="R69" s="289"/>
-      <c r="S69" s="289"/>
+      <c r="I69" s="235"/>
+      <c r="P69" s="246"/>
+      <c r="Q69" s="246"/>
+      <c r="R69" s="209"/>
+      <c r="S69" s="209"/>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A70" s="86"/>
@@ -7688,68 +7699,68 @@
       <c r="F70" t="s">
         <v>60</v>
       </c>
-      <c r="H70" s="293">
+      <c r="H70" s="247">
         <v>5.5410000000000004</v>
       </c>
-      <c r="I70" s="293"/>
-      <c r="P70" s="288"/>
-      <c r="Q70" s="288"/>
-      <c r="R70" s="289"/>
-      <c r="S70" s="289"/>
+      <c r="I70" s="247"/>
+      <c r="P70" s="246"/>
+      <c r="Q70" s="246"/>
+      <c r="R70" s="209"/>
+      <c r="S70" s="209"/>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A71" s="86"/>
       <c r="F71" t="s">
         <v>62</v>
       </c>
-      <c r="H71" s="287">
+      <c r="H71" s="248">
         <v>11.78</v>
       </c>
-      <c r="I71" s="287"/>
-      <c r="P71" s="288"/>
-      <c r="Q71" s="288"/>
-      <c r="R71" s="289"/>
-      <c r="S71" s="289"/>
+      <c r="I71" s="248"/>
+      <c r="P71" s="246"/>
+      <c r="Q71" s="246"/>
+      <c r="R71" s="209"/>
+      <c r="S71" s="209"/>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A72" s="86"/>
       <c r="F72" t="s">
         <v>65</v>
       </c>
-      <c r="H72" s="287">
+      <c r="H72" s="248">
         <v>12.39</v>
       </c>
-      <c r="I72" s="287"/>
-      <c r="P72" s="288"/>
-      <c r="Q72" s="288"/>
-      <c r="R72" s="289"/>
-      <c r="S72" s="289"/>
+      <c r="I72" s="248"/>
+      <c r="P72" s="246"/>
+      <c r="Q72" s="246"/>
+      <c r="R72" s="209"/>
+      <c r="S72" s="209"/>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A73" s="86"/>
       <c r="F73" t="s">
         <v>207</v>
       </c>
-      <c r="H73" s="287">
+      <c r="H73" s="248">
         <v>11.21</v>
       </c>
-      <c r="I73" s="287"/>
+      <c r="I73" s="248"/>
       <c r="J73" s="88"/>
       <c r="K73" s="88"/>
-      <c r="P73" s="288"/>
-      <c r="Q73" s="288"/>
-      <c r="R73" s="289"/>
-      <c r="S73" s="289"/>
+      <c r="P73" s="246"/>
+      <c r="Q73" s="246"/>
+      <c r="R73" s="209"/>
+      <c r="S73" s="209"/>
     </row>
     <row r="74" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A74" s="86"/>
       <c r="F74" t="s">
         <v>208</v>
       </c>
-      <c r="H74" s="290">
+      <c r="H74" s="249">
         <v>12.75</v>
       </c>
-      <c r="I74" s="290"/>
+      <c r="I74" s="249"/>
       <c r="J74" s="95">
         <f>AVERAGE(H71:I74)</f>
         <v>12.032500000000001</v>
@@ -7758,28 +7769,28 @@
         <f>ABS(H75-D75)/D75*100</f>
         <v>4.2097852868708063</v>
       </c>
-      <c r="P74" s="288"/>
-      <c r="Q74" s="288"/>
-      <c r="R74" s="289"/>
-      <c r="S74" s="289"/>
+      <c r="P74" s="246"/>
+      <c r="Q74" s="246"/>
+      <c r="R74" s="209"/>
+      <c r="S74" s="209"/>
     </row>
     <row r="75" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="96"/>
-      <c r="B75" s="277" t="s">
+      <c r="B75" s="216" t="s">
         <v>209</v>
       </c>
-      <c r="C75" s="278"/>
+      <c r="C75" s="217"/>
       <c r="D75" s="91">
         <v>9.4700000000000006</v>
       </c>
       <c r="E75" s="97"/>
       <c r="F75" s="97"/>
       <c r="G75" s="97"/>
-      <c r="H75" s="279">
+      <c r="H75" s="260">
         <f>(H70/3)+(2/3*J74)</f>
         <v>9.868666666666666</v>
       </c>
-      <c r="I75" s="280"/>
+      <c r="I75" s="261"/>
       <c r="J75" s="98"/>
       <c r="K75" s="98"/>
     </row>
@@ -7787,24 +7798,24 @@
       <c r="G76" s="99" t="s">
         <v>39</v>
       </c>
-      <c r="H76" s="180" t="str">
+      <c r="H76" s="223" t="str">
         <f>IF(K74&lt;20,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I76" s="182"/>
+      <c r="I76" s="262"/>
     </row>
     <row r="77" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="281" t="s">
+      <c r="A77" s="263" t="s">
         <v>212</v>
       </c>
-      <c r="B77" s="282"/>
-      <c r="C77" s="282"/>
-      <c r="D77" s="282"/>
-      <c r="E77" s="282"/>
-      <c r="F77" s="282"/>
-      <c r="G77" s="282"/>
-      <c r="H77" s="282"/>
-      <c r="I77" s="283"/>
+      <c r="B77" s="264"/>
+      <c r="C77" s="264"/>
+      <c r="D77" s="264"/>
+      <c r="E77" s="264"/>
+      <c r="F77" s="264"/>
+      <c r="G77" s="264"/>
+      <c r="H77" s="264"/>
+      <c r="I77" s="265"/>
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.3">
       <c r="G78" s="9"/>
@@ -7817,11 +7828,11 @@
       <c r="I79" s="100"/>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A80" s="180" t="s">
+      <c r="A80" s="223" t="s">
         <v>213</v>
       </c>
-      <c r="B80" s="181"/>
-      <c r="C80" s="181"/>
+      <c r="B80" s="266"/>
+      <c r="C80" s="266"/>
       <c r="D80" s="47" t="s">
         <v>214</v>
       </c>
@@ -7838,10 +7849,10 @@
       <c r="A81" s="101" t="s">
         <v>41</v>
       </c>
-      <c r="B81" s="284" t="s">
+      <c r="B81" s="267" t="s">
         <v>4</v>
       </c>
-      <c r="C81" s="285"/>
+      <c r="C81" s="268"/>
       <c r="D81" s="102" t="s">
         <v>216</v>
       </c>
@@ -7850,8 +7861,8 @@
         <v>0.5</v>
       </c>
       <c r="G81" s="88"/>
-      <c r="H81" s="286"/>
-      <c r="I81" s="286"/>
+      <c r="H81" s="269"/>
+      <c r="I81" s="269"/>
       <c r="J81" s="88"/>
       <c r="K81" s="88"/>
     </row>
@@ -7859,11 +7870,11 @@
       <c r="A82" s="104">
         <v>140</v>
       </c>
-      <c r="B82" s="268">
+      <c r="B82" s="250">
         <v>15</v>
       </c>
-      <c r="C82" s="268"/>
-      <c r="D82" s="269" t="s">
+      <c r="C82" s="250"/>
+      <c r="D82" s="251" t="s">
         <v>217</v>
       </c>
       <c r="E82" s="106"/>
@@ -7881,11 +7892,11 @@
       <c r="A83" s="50" t="s">
         <v>219</v>
       </c>
-      <c r="B83" s="272" t="s">
+      <c r="B83" s="254" t="s">
         <v>220</v>
       </c>
-      <c r="C83" s="263"/>
-      <c r="D83" s="270"/>
+      <c r="C83" s="255"/>
+      <c r="D83" s="252"/>
       <c r="E83" s="46" t="s">
         <v>221</v>
       </c>
@@ -7906,11 +7917,11 @@
       <c r="A84" s="50">
         <v>1.25</v>
       </c>
-      <c r="B84" s="273">
+      <c r="B84" s="256">
         <v>2.8</v>
       </c>
-      <c r="C84" s="273"/>
-      <c r="D84" s="270"/>
+      <c r="C84" s="256"/>
+      <c r="D84" s="252"/>
       <c r="E84" s="111">
         <f>B84*E81</f>
         <v>1.4</v>
@@ -7936,11 +7947,11 @@
       <c r="A85" s="50">
         <v>2.5</v>
       </c>
-      <c r="B85" s="274">
+      <c r="B85" s="257">
         <v>5</v>
       </c>
-      <c r="C85" s="275"/>
-      <c r="D85" s="270"/>
+      <c r="C85" s="258"/>
+      <c r="D85" s="252"/>
       <c r="E85" s="111">
         <f>B85*E81</f>
         <v>2.5</v>
@@ -7962,11 +7973,11 @@
       <c r="A86" s="113">
         <v>5</v>
       </c>
-      <c r="B86" s="276">
+      <c r="B86" s="259">
         <v>9.8000000000000007</v>
       </c>
-      <c r="C86" s="276"/>
-      <c r="D86" s="271"/>
+      <c r="C86" s="259"/>
+      <c r="D86" s="253"/>
       <c r="E86" s="115">
         <f>B86*E81</f>
         <v>4.9000000000000004</v>
@@ -7985,14 +7996,14 @@
       <c r="K86" s="88"/>
     </row>
     <row r="87" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="254" t="s">
+      <c r="A87" s="282" t="s">
         <v>223</v>
       </c>
-      <c r="B87" s="255"/>
-      <c r="C87" s="255"/>
-      <c r="D87" s="255"/>
-      <c r="E87" s="255"/>
-      <c r="F87" s="256"/>
+      <c r="B87" s="283"/>
+      <c r="C87" s="283"/>
+      <c r="D87" s="283"/>
+      <c r="E87" s="283"/>
+      <c r="F87" s="284"/>
       <c r="G87" s="88"/>
       <c r="H87" s="88"/>
       <c r="I87" s="88"/>
@@ -8000,12 +8011,12 @@
       <c r="K87" s="88"/>
     </row>
     <row r="88" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="257"/>
-      <c r="B88" s="258"/>
-      <c r="C88" s="258"/>
-      <c r="D88" s="258"/>
-      <c r="E88" s="258"/>
-      <c r="F88" s="259"/>
+      <c r="A88" s="285"/>
+      <c r="B88" s="286"/>
+      <c r="C88" s="286"/>
+      <c r="D88" s="286"/>
+      <c r="E88" s="286"/>
+      <c r="F88" s="287"/>
       <c r="G88" s="88"/>
       <c r="H88" s="88"/>
       <c r="I88" s="88"/>
@@ -8020,11 +8031,11 @@
       <c r="B90" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="C90" s="181" t="s">
+      <c r="C90" s="266" t="s">
         <v>224</v>
       </c>
-      <c r="D90" s="181"/>
-      <c r="E90" s="182"/>
+      <c r="D90" s="266"/>
+      <c r="E90" s="262"/>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91" s="118">
@@ -8036,37 +8047,37 @@
       <c r="C91" s="119" t="s">
         <v>106</v>
       </c>
-      <c r="D91" s="260">
+      <c r="D91" s="288">
         <v>107</v>
       </c>
-      <c r="E91" s="261"/>
+      <c r="E91" s="289"/>
       <c r="F91" s="120" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A92" s="262" t="s">
+      <c r="A92" s="290" t="s">
         <v>225</v>
       </c>
-      <c r="B92" s="263"/>
-      <c r="C92" s="264">
+      <c r="B92" s="255"/>
+      <c r="C92" s="291">
         <v>3</v>
       </c>
-      <c r="D92" s="264"/>
-      <c r="E92" s="264"/>
+      <c r="D92" s="291"/>
+      <c r="E92" s="291"/>
       <c r="F92" s="121" t="str">
         <f>IF(C92&lt;=5,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A93" s="265" t="s">
+      <c r="A93" s="292" t="s">
         <v>226</v>
       </c>
-      <c r="B93" s="266"/>
-      <c r="C93" s="266"/>
-      <c r="D93" s="266"/>
-      <c r="E93" s="267"/>
+      <c r="B93" s="293"/>
+      <c r="C93" s="293"/>
+      <c r="D93" s="293"/>
+      <c r="E93" s="294"/>
     </row>
     <row r="94" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A94" s="122"/>
@@ -8082,11 +8093,11 @@
       <c r="B95" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="C95" s="242" t="s">
+      <c r="C95" s="244" t="s">
         <v>227</v>
       </c>
-      <c r="D95" s="243"/>
-      <c r="E95" s="244"/>
+      <c r="D95" s="270"/>
+      <c r="E95" s="245"/>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96" s="118">
@@ -8098,44 +8109,44 @@
       <c r="C96" s="127" t="s">
         <v>106</v>
       </c>
-      <c r="D96" s="245">
+      <c r="D96" s="271">
         <v>3691</v>
       </c>
-      <c r="E96" s="246"/>
+      <c r="E96" s="272"/>
       <c r="F96" s="120" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="97" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="247" t="s">
+      <c r="A97" s="273" t="s">
         <v>225</v>
       </c>
-      <c r="B97" s="248"/>
-      <c r="C97" s="249">
+      <c r="B97" s="274"/>
+      <c r="C97" s="275">
         <v>6.25</v>
       </c>
-      <c r="D97" s="249"/>
-      <c r="E97" s="249"/>
+      <c r="D97" s="275"/>
+      <c r="E97" s="275"/>
       <c r="F97" s="121" t="str">
         <f>IF(C97&gt;=3.12,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A98" s="250" t="s">
+      <c r="A98" s="276" t="s">
         <v>228</v>
       </c>
-      <c r="B98" s="251"/>
-      <c r="C98" s="251"/>
-      <c r="D98" s="251"/>
-      <c r="E98" s="252"/>
+      <c r="B98" s="277"/>
+      <c r="C98" s="277"/>
+      <c r="D98" s="277"/>
+      <c r="E98" s="278"/>
     </row>
     <row r="99" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="225"/>
-      <c r="B99" s="253"/>
-      <c r="C99" s="253"/>
-      <c r="D99" s="253"/>
-      <c r="E99" s="226"/>
+      <c r="A99" s="279"/>
+      <c r="B99" s="280"/>
+      <c r="C99" s="280"/>
+      <c r="D99" s="280"/>
+      <c r="E99" s="281"/>
     </row>
     <row r="100" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="128"/>
@@ -8145,18 +8156,18 @@
       <c r="E100" s="128"/>
     </row>
     <row r="101" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="242" t="s">
+      <c r="A101" s="244" t="s">
         <v>229</v>
       </c>
-      <c r="B101" s="243"/>
-      <c r="C101" s="243"/>
-      <c r="D101" s="243"/>
-      <c r="E101" s="243"/>
-      <c r="F101" s="243"/>
-      <c r="G101" s="243"/>
-      <c r="H101" s="243"/>
-      <c r="I101" s="243"/>
-      <c r="J101" s="244"/>
+      <c r="B101" s="270"/>
+      <c r="C101" s="270"/>
+      <c r="D101" s="270"/>
+      <c r="E101" s="270"/>
+      <c r="F101" s="270"/>
+      <c r="G101" s="270"/>
+      <c r="H101" s="270"/>
+      <c r="I101" s="270"/>
+      <c r="J101" s="245"/>
     </row>
     <row r="102" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A102" s="89" t="s">
@@ -8179,8 +8190,8 @@
         <v>232</v>
       </c>
       <c r="H102" s="130"/>
-      <c r="I102" s="219"/>
-      <c r="J102" s="220"/>
+      <c r="I102" s="300"/>
+      <c r="J102" s="301"/>
     </row>
     <row r="103" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A103" s="131">
@@ -8192,24 +8203,24 @@
       <c r="C103" s="133">
         <v>1</v>
       </c>
-      <c r="D103" s="221"/>
-      <c r="E103" s="222"/>
-      <c r="F103" s="222"/>
-      <c r="G103" s="223" t="s">
+      <c r="D103" s="302"/>
+      <c r="E103" s="178"/>
+      <c r="F103" s="178"/>
+      <c r="G103" s="303" t="s">
         <v>233</v>
       </c>
-      <c r="H103" s="224"/>
-      <c r="I103" s="227" t="s">
+      <c r="H103" s="304"/>
+      <c r="I103" s="305" t="s">
         <v>234</v>
       </c>
-      <c r="J103" s="228"/>
-      <c r="K103" s="231" t="s">
+      <c r="J103" s="306"/>
+      <c r="K103" s="307" t="s">
         <v>39</v>
       </c>
-      <c r="L103" s="232"/>
+      <c r="L103" s="308"/>
     </row>
     <row r="104" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A104" s="235" t="s">
+      <c r="A104" s="311" t="s">
         <v>96</v>
       </c>
       <c r="B104" s="134" t="s">
@@ -8227,15 +8238,15 @@
       <c r="F104" s="135" t="s">
         <v>239</v>
       </c>
-      <c r="G104" s="225"/>
-      <c r="H104" s="226"/>
-      <c r="I104" s="229"/>
+      <c r="G104" s="279"/>
+      <c r="H104" s="281"/>
+      <c r="I104" s="228"/>
       <c r="J104" s="230"/>
-      <c r="K104" s="233"/>
-      <c r="L104" s="234"/>
+      <c r="K104" s="309"/>
+      <c r="L104" s="310"/>
     </row>
     <row r="105" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A105" s="194"/>
+      <c r="A105" s="312"/>
       <c r="B105" s="138"/>
       <c r="C105" s="139"/>
       <c r="D105" s="139"/>
@@ -8243,37 +8254,37 @@
       <c r="F105" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="G105" s="236">
+      <c r="G105" s="313">
         <f>ROUND(F102*MAX(B105:E105)/(60*B103),3)</f>
         <v>0</v>
       </c>
-      <c r="H105" s="237"/>
-      <c r="I105" s="238">
+      <c r="H105" s="314"/>
+      <c r="I105" s="315">
         <f>ROUND(8.33*MAX(B105:F105)/(B103*114),3)</f>
         <v>0</v>
       </c>
-      <c r="J105" s="239"/>
-      <c r="K105" s="240" t="str">
+      <c r="J105" s="316"/>
+      <c r="K105" s="317" t="str">
         <f>IF(I105&lt;=1,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="L105" s="241"/>
+      <c r="L105" s="318"/>
     </row>
     <row r="106" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A106" s="210" t="s">
+      <c r="A106" s="220" t="s">
         <v>240</v>
       </c>
-      <c r="B106" s="211"/>
-      <c r="C106" s="211"/>
-      <c r="D106" s="211"/>
-      <c r="E106" s="211"/>
-      <c r="F106" s="211"/>
-      <c r="G106" s="211"/>
-      <c r="H106" s="211"/>
-      <c r="I106" s="211"/>
-      <c r="J106" s="211"/>
-      <c r="K106" s="211"/>
-      <c r="L106" s="212"/>
+      <c r="B106" s="221"/>
+      <c r="C106" s="221"/>
+      <c r="D106" s="221"/>
+      <c r="E106" s="221"/>
+      <c r="F106" s="221"/>
+      <c r="G106" s="221"/>
+      <c r="H106" s="221"/>
+      <c r="I106" s="221"/>
+      <c r="J106" s="221"/>
+      <c r="K106" s="221"/>
+      <c r="L106" s="222"/>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
@@ -8322,44 +8333,44 @@
       <c r="I112" s="88"/>
     </row>
     <row r="113" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="213" t="s">
+      <c r="A113" s="295" t="s">
         <v>87</v>
       </c>
-      <c r="B113" s="214"/>
-      <c r="C113" s="214"/>
-      <c r="D113" s="214"/>
-      <c r="E113" s="214" t="s">
+      <c r="B113" s="296"/>
+      <c r="C113" s="296"/>
+      <c r="D113" s="296"/>
+      <c r="E113" s="296" t="s">
         <v>244</v>
       </c>
-      <c r="F113" s="214"/>
-      <c r="G113" s="214" t="s">
+      <c r="F113" s="296"/>
+      <c r="G113" s="296" t="s">
         <v>245</v>
       </c>
-      <c r="H113" s="214" t="s">
+      <c r="H113" s="296" t="s">
         <v>39</v>
       </c>
-      <c r="I113" s="217" t="s">
+      <c r="I113" s="298" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="114" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="215"/>
-      <c r="B114" s="216"/>
-      <c r="C114" s="216"/>
-      <c r="D114" s="216"/>
-      <c r="E114" s="216"/>
-      <c r="F114" s="216"/>
-      <c r="G114" s="216"/>
-      <c r="H114" s="216"/>
-      <c r="I114" s="218"/>
+      <c r="A114" s="297"/>
+      <c r="B114" s="188"/>
+      <c r="C114" s="188"/>
+      <c r="D114" s="188"/>
+      <c r="E114" s="188"/>
+      <c r="F114" s="188"/>
+      <c r="G114" s="188"/>
+      <c r="H114" s="188"/>
+      <c r="I114" s="299"/>
     </row>
     <row r="115" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="205" t="s">
+      <c r="A115" s="326" t="s">
         <v>247</v>
       </c>
-      <c r="B115" s="206"/>
-      <c r="C115" s="206"/>
-      <c r="D115" s="206"/>
+      <c r="B115" s="327"/>
+      <c r="C115" s="327"/>
+      <c r="D115" s="327"/>
       <c r="E115" s="144">
         <v>2.7E-2</v>
       </c>
@@ -8374,17 +8385,17 @@
         <f>IF(E115&lt;=2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I115" s="207" t="s">
+      <c r="I115" s="328" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="116" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="201" t="s">
+      <c r="A116" s="322" t="s">
         <v>249</v>
       </c>
-      <c r="B116" s="202"/>
-      <c r="C116" s="202"/>
-      <c r="D116" s="202"/>
+      <c r="B116" s="323"/>
+      <c r="C116" s="323"/>
+      <c r="D116" s="323"/>
       <c r="E116" s="148">
         <v>4.3999999999999997E-2</v>
       </c>
@@ -8399,15 +8410,15 @@
         <f t="shared" ref="H116:H119" si="11">IF(E116&lt;=2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I116" s="208"/>
+      <c r="I116" s="329"/>
     </row>
     <row r="117" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="201" t="s">
+      <c r="A117" s="322" t="s">
         <v>250</v>
       </c>
-      <c r="B117" s="202"/>
-      <c r="C117" s="202"/>
-      <c r="D117" s="202"/>
+      <c r="B117" s="323"/>
+      <c r="C117" s="323"/>
+      <c r="D117" s="323"/>
       <c r="E117" s="148">
         <v>3.4000000000000002E-2</v>
       </c>
@@ -8422,15 +8433,15 @@
         <f t="shared" si="11"/>
         <v>Pass</v>
       </c>
-      <c r="I117" s="208"/>
+      <c r="I117" s="329"/>
     </row>
     <row r="118" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="201" t="s">
+      <c r="A118" s="322" t="s">
         <v>251</v>
       </c>
-      <c r="B118" s="202"/>
-      <c r="C118" s="202"/>
-      <c r="D118" s="202"/>
+      <c r="B118" s="323"/>
+      <c r="C118" s="323"/>
+      <c r="D118" s="323"/>
       <c r="E118" s="148">
         <v>0.04</v>
       </c>
@@ -8445,15 +8456,15 @@
         <f t="shared" si="11"/>
         <v>Pass</v>
       </c>
-      <c r="I118" s="208"/>
+      <c r="I118" s="329"/>
     </row>
     <row r="119" spans="1:15" ht="14.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A119" s="203" t="s">
+      <c r="A119" s="324" t="s">
         <v>252</v>
       </c>
-      <c r="B119" s="204"/>
-      <c r="C119" s="204"/>
-      <c r="D119" s="204"/>
+      <c r="B119" s="325"/>
+      <c r="C119" s="325"/>
+      <c r="D119" s="325"/>
       <c r="E119" s="150">
         <v>3.2000000000000001E-2</v>
       </c>
@@ -8468,15 +8479,15 @@
         <f t="shared" si="11"/>
         <v>Pass</v>
       </c>
-      <c r="I119" s="209"/>
+      <c r="I119" s="330"/>
     </row>
     <row r="120" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="196" t="s">
+      <c r="A120" s="345" t="s">
         <v>253</v>
       </c>
-      <c r="B120" s="197"/>
-      <c r="C120" s="197"/>
-      <c r="D120" s="197"/>
+      <c r="B120" s="346"/>
+      <c r="C120" s="346"/>
+      <c r="D120" s="346"/>
       <c r="E120" s="154">
         <v>0.106</v>
       </c>
@@ -8491,17 +8502,17 @@
         <f>IF(E120&lt;=0.2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I120" s="198" t="s">
+      <c r="I120" s="319" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="121" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="201" t="s">
+      <c r="A121" s="322" t="s">
         <v>255</v>
       </c>
-      <c r="B121" s="202"/>
-      <c r="C121" s="202"/>
-      <c r="D121" s="202"/>
+      <c r="B121" s="323"/>
+      <c r="C121" s="323"/>
+      <c r="D121" s="323"/>
       <c r="E121" s="148">
         <v>3.7999999999999999E-2</v>
       </c>
@@ -8516,15 +8527,15 @@
         <f t="shared" ref="H121:H123" si="12">IF(E121&lt;=0.2,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="I121" s="199"/>
+      <c r="I121" s="320"/>
     </row>
     <row r="122" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="201" t="s">
+      <c r="A122" s="322" t="s">
         <v>256</v>
       </c>
-      <c r="B122" s="202"/>
-      <c r="C122" s="202"/>
-      <c r="D122" s="202"/>
+      <c r="B122" s="323"/>
+      <c r="C122" s="323"/>
+      <c r="D122" s="323"/>
       <c r="E122" s="148">
         <v>4.2000000000000003E-2</v>
       </c>
@@ -8539,15 +8550,15 @@
         <f t="shared" si="12"/>
         <v>Pass</v>
       </c>
-      <c r="I122" s="199"/>
+      <c r="I122" s="320"/>
     </row>
     <row r="123" spans="1:15" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="201" t="s">
+      <c r="A123" s="322" t="s">
         <v>257</v>
       </c>
-      <c r="B123" s="202"/>
-      <c r="C123" s="202"/>
-      <c r="D123" s="202"/>
+      <c r="B123" s="323"/>
+      <c r="C123" s="323"/>
+      <c r="D123" s="323"/>
       <c r="E123" s="148">
         <v>2.4E-2</v>
       </c>
@@ -8562,15 +8573,15 @@
         <f t="shared" si="12"/>
         <v>Pass</v>
       </c>
-      <c r="I123" s="199"/>
+      <c r="I123" s="320"/>
     </row>
     <row r="124" spans="1:15" ht="14.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A124" s="203" t="s">
+      <c r="A124" s="324" t="s">
         <v>258</v>
       </c>
-      <c r="B124" s="204"/>
-      <c r="C124" s="204"/>
-      <c r="D124" s="204"/>
+      <c r="B124" s="325"/>
+      <c r="C124" s="325"/>
+      <c r="D124" s="325"/>
       <c r="E124" s="150"/>
       <c r="F124" s="151" t="s">
         <v>128</v>
@@ -8581,7 +8592,7 @@
       <c r="H124" s="153" t="s">
         <v>259</v>
       </c>
-      <c r="I124" s="200"/>
+      <c r="I124" s="321"/>
     </row>
     <row r="125" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H125" s="88"/>
@@ -8602,15 +8613,15 @@
       <c r="I126" s="88"/>
     </row>
     <row r="127" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A127" s="180" t="s">
+      <c r="A127" s="223" t="s">
         <v>262</v>
       </c>
-      <c r="B127" s="181"/>
-      <c r="C127" s="181"/>
-      <c r="D127" s="181"/>
-      <c r="E127" s="181"/>
-      <c r="F127" s="181"/>
-      <c r="G127" s="182"/>
+      <c r="B127" s="266"/>
+      <c r="C127" s="266"/>
+      <c r="D127" s="266"/>
+      <c r="E127" s="266"/>
+      <c r="F127" s="266"/>
+      <c r="G127" s="262"/>
       <c r="H127" s="98"/>
       <c r="I127" s="98"/>
       <c r="J127" s="98"/>
@@ -8624,12 +8635,12 @@
       <c r="A128" s="99" t="s">
         <v>263</v>
       </c>
-      <c r="B128" s="183" t="s">
+      <c r="B128" s="194" t="s">
         <v>264</v>
       </c>
-      <c r="C128" s="184"/>
-      <c r="D128" s="184"/>
-      <c r="E128" s="185"/>
+      <c r="C128" s="195"/>
+      <c r="D128" s="195"/>
+      <c r="E128" s="196"/>
       <c r="F128" s="162" t="s">
         <v>265</v>
       </c>
@@ -8716,15 +8727,15 @@
       <c r="O130" s="98"/>
     </row>
     <row r="131" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A131" s="186" t="s">
+      <c r="A131" s="336" t="s">
         <v>270</v>
       </c>
-      <c r="B131" s="176"/>
-      <c r="C131" s="176"/>
-      <c r="D131" s="176"/>
-      <c r="E131" s="176"/>
-      <c r="F131" s="176"/>
-      <c r="G131" s="177"/>
+      <c r="B131" s="332"/>
+      <c r="C131" s="332"/>
+      <c r="D131" s="332"/>
+      <c r="E131" s="332"/>
+      <c r="F131" s="332"/>
+      <c r="G131" s="333"/>
       <c r="H131" s="88"/>
       <c r="I131" s="88"/>
       <c r="J131" s="88"/>
@@ -8735,15 +8746,15 @@
       <c r="O131" s="98"/>
     </row>
     <row r="132" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="187" t="s">
+      <c r="A132" s="337" t="s">
         <v>271</v>
       </c>
-      <c r="B132" s="188"/>
-      <c r="C132" s="188"/>
-      <c r="D132" s="188"/>
-      <c r="E132" s="188"/>
-      <c r="F132" s="188"/>
-      <c r="G132" s="189"/>
+      <c r="B132" s="338"/>
+      <c r="C132" s="338"/>
+      <c r="D132" s="338"/>
+      <c r="E132" s="338"/>
+      <c r="F132" s="338"/>
+      <c r="G132" s="339"/>
       <c r="H132" s="88"/>
       <c r="I132" s="88"/>
       <c r="J132" s="88"/>
@@ -8754,13 +8765,13 @@
       <c r="O132" s="98"/>
     </row>
     <row r="133" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A133" s="190"/>
-      <c r="B133" s="191"/>
-      <c r="C133" s="191"/>
-      <c r="D133" s="191"/>
-      <c r="E133" s="191"/>
-      <c r="F133" s="191"/>
-      <c r="G133" s="192"/>
+      <c r="A133" s="340"/>
+      <c r="B133" s="341"/>
+      <c r="C133" s="341"/>
+      <c r="D133" s="341"/>
+      <c r="E133" s="341"/>
+      <c r="F133" s="341"/>
+      <c r="G133" s="342"/>
       <c r="H133" s="98"/>
       <c r="I133" s="98"/>
       <c r="J133" s="98"/>
@@ -8867,7 +8878,7 @@
       <c r="O139" s="98"/>
     </row>
     <row r="140" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A140" s="193" t="s">
+      <c r="A140" s="343" t="s">
         <v>2</v>
       </c>
       <c r="B140" s="20">
@@ -8898,7 +8909,7 @@
       <c r="O140" s="98"/>
     </row>
     <row r="141" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A141" s="194"/>
+      <c r="A141" s="312"/>
       <c r="B141" s="20">
         <f>B140-B140</f>
         <v>0</v>
@@ -8934,7 +8945,7 @@
     </row>
     <row r="142" spans="1:15" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="96"/>
-      <c r="B142" s="195" t="s">
+      <c r="B142" s="344" t="s">
         <v>275</v>
       </c>
       <c r="C142" s="173">
@@ -8968,7 +8979,7 @@
     </row>
     <row r="143" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="96"/>
-      <c r="B143" s="195"/>
+      <c r="B143" s="344"/>
       <c r="C143" s="20" t="str">
         <f t="shared" ref="C143:E143" si="14">IF(C142&gt;1,"Fail","Pass")</f>
         <v>Pass</v>
@@ -8999,26 +9010,26 @@
       <c r="O143" s="98"/>
     </row>
     <row r="144" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A144" s="175" t="s">
+      <c r="A144" s="331" t="s">
         <v>276</v>
       </c>
-      <c r="B144" s="176"/>
-      <c r="C144" s="176"/>
-      <c r="D144" s="176"/>
-      <c r="E144" s="176"/>
-      <c r="F144" s="176"/>
-      <c r="G144" s="177"/>
+      <c r="B144" s="332"/>
+      <c r="C144" s="332"/>
+      <c r="D144" s="332"/>
+      <c r="E144" s="332"/>
+      <c r="F144" s="332"/>
+      <c r="G144" s="333"/>
     </row>
     <row r="145" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A145" s="175" t="s">
+      <c r="A145" s="331" t="s">
         <v>277</v>
       </c>
-      <c r="B145" s="178"/>
-      <c r="C145" s="178"/>
-      <c r="D145" s="178"/>
-      <c r="E145" s="178"/>
-      <c r="F145" s="178"/>
-      <c r="G145" s="179"/>
+      <c r="B145" s="334"/>
+      <c r="C145" s="334"/>
+      <c r="D145" s="334"/>
+      <c r="E145" s="334"/>
+      <c r="F145" s="334"/>
+      <c r="G145" s="335"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -9034,107 +9045,26 @@
     <protectedRange sqref="A126" name="Range10"/>
   </protectedRanges>
   <mergeCells count="136">
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="P11:X11"/>
-    <mergeCell ref="P12:P13"/>
-    <mergeCell ref="Q12:S12"/>
-    <mergeCell ref="T12:T13"/>
-    <mergeCell ref="U12:U13"/>
-    <mergeCell ref="V12:V13"/>
-    <mergeCell ref="X12:X13"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B10:I10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="P25:U25"/>
-    <mergeCell ref="P27:R27"/>
-    <mergeCell ref="P18:V18"/>
-    <mergeCell ref="P19:V19"/>
-    <mergeCell ref="P20:U20"/>
-    <mergeCell ref="P21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="H65:I65"/>
-    <mergeCell ref="P41:Y41"/>
-    <mergeCell ref="P43:Q43"/>
-    <mergeCell ref="P45:S47"/>
-    <mergeCell ref="A57:I57"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="Q28:S28"/>
-    <mergeCell ref="U29:U32"/>
-    <mergeCell ref="X29:X32"/>
-    <mergeCell ref="P33:X33"/>
-    <mergeCell ref="P35:Y35"/>
-    <mergeCell ref="Q36:U36"/>
-    <mergeCell ref="H66:I66"/>
-    <mergeCell ref="H69:I69"/>
-    <mergeCell ref="P69:Q69"/>
-    <mergeCell ref="R69:S69"/>
-    <mergeCell ref="H70:I70"/>
-    <mergeCell ref="P70:Q70"/>
-    <mergeCell ref="R70:S70"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="H62:I62"/>
-    <mergeCell ref="H63:I63"/>
-    <mergeCell ref="H64:I64"/>
-    <mergeCell ref="H73:I73"/>
-    <mergeCell ref="P73:Q73"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="H74:I74"/>
-    <mergeCell ref="P74:Q74"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="H71:I71"/>
-    <mergeCell ref="P71:Q71"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="H72:I72"/>
-    <mergeCell ref="P72:Q72"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="D82:D86"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="H75:I75"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="A77:I77"/>
-    <mergeCell ref="A80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="H81:I81"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="D96:E96"/>
-    <mergeCell ref="A97:B97"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="A98:E99"/>
-    <mergeCell ref="A101:J101"/>
-    <mergeCell ref="A87:F88"/>
-    <mergeCell ref="C90:E90"/>
-    <mergeCell ref="D91:E91"/>
-    <mergeCell ref="A92:B92"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A144:G144"/>
+    <mergeCell ref="A145:G145"/>
+    <mergeCell ref="A127:G127"/>
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="A131:G131"/>
+    <mergeCell ref="A132:G133"/>
+    <mergeCell ref="A140:A141"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="A120:D120"/>
+    <mergeCell ref="I120:I124"/>
+    <mergeCell ref="A121:D121"/>
+    <mergeCell ref="A122:D122"/>
+    <mergeCell ref="A123:D123"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="I115:I119"/>
+    <mergeCell ref="A116:D116"/>
+    <mergeCell ref="A117:D117"/>
+    <mergeCell ref="A118:D118"/>
+    <mergeCell ref="A119:D119"/>
     <mergeCell ref="A106:L106"/>
     <mergeCell ref="A113:D114"/>
     <mergeCell ref="E113:F114"/>
@@ -9150,26 +9080,107 @@
     <mergeCell ref="G105:H105"/>
     <mergeCell ref="I105:J105"/>
     <mergeCell ref="K105:L105"/>
-    <mergeCell ref="I120:I124"/>
-    <mergeCell ref="A121:D121"/>
-    <mergeCell ref="A122:D122"/>
-    <mergeCell ref="A123:D123"/>
-    <mergeCell ref="A124:D124"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="I115:I119"/>
-    <mergeCell ref="A116:D116"/>
-    <mergeCell ref="A117:D117"/>
-    <mergeCell ref="A118:D118"/>
-    <mergeCell ref="A119:D119"/>
-    <mergeCell ref="A144:G144"/>
-    <mergeCell ref="A145:G145"/>
-    <mergeCell ref="A127:G127"/>
-    <mergeCell ref="B128:E128"/>
-    <mergeCell ref="A131:G131"/>
-    <mergeCell ref="A132:G133"/>
-    <mergeCell ref="A140:A141"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="A120:D120"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="D96:E96"/>
+    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="A98:E99"/>
+    <mergeCell ref="A101:J101"/>
+    <mergeCell ref="A87:F88"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="D91:E91"/>
+    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="D82:D86"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="H75:I75"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="A80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="H81:I81"/>
+    <mergeCell ref="H73:I73"/>
+    <mergeCell ref="P73:Q73"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="H74:I74"/>
+    <mergeCell ref="P74:Q74"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="H71:I71"/>
+    <mergeCell ref="P71:Q71"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="H72:I72"/>
+    <mergeCell ref="P72:Q72"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="H66:I66"/>
+    <mergeCell ref="H69:I69"/>
+    <mergeCell ref="P69:Q69"/>
+    <mergeCell ref="R69:S69"/>
+    <mergeCell ref="H70:I70"/>
+    <mergeCell ref="P70:Q70"/>
+    <mergeCell ref="R70:S70"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="H62:I62"/>
+    <mergeCell ref="H63:I63"/>
+    <mergeCell ref="H64:I64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="H65:I65"/>
+    <mergeCell ref="P41:Y41"/>
+    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="P45:S47"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="Q28:S28"/>
+    <mergeCell ref="U29:U32"/>
+    <mergeCell ref="X29:X32"/>
+    <mergeCell ref="P33:X33"/>
+    <mergeCell ref="P35:Y35"/>
+    <mergeCell ref="Q36:U36"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="P25:U25"/>
+    <mergeCell ref="P27:R27"/>
+    <mergeCell ref="P18:V18"/>
+    <mergeCell ref="P19:V19"/>
+    <mergeCell ref="P20:U20"/>
+    <mergeCell ref="P21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="P11:X11"/>
+    <mergeCell ref="P12:P13"/>
+    <mergeCell ref="Q12:S12"/>
+    <mergeCell ref="T12:T13"/>
+    <mergeCell ref="U12:U13"/>
+    <mergeCell ref="V12:V13"/>
+    <mergeCell ref="X12:X13"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B4:I4"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="C142:G142">

</xml_diff>